<commit_message>
Task completed: Answered the user's question: the route-gap bug should no longer recur after the updated code runs its route sync, but other missing/inactive reviewer assignments can still block forwarding. Live database/browser verification was unavailable, so this is not a guarantee.
</commit_message>
<xml_diff>
--- a/Raquel_Pawnshop_HR_Workforce_Analytics_&_Evaluation _Platform-Computation.xlsx
+++ b/Raquel_Pawnshop_HR_Workforce_Analytics_&_Evaluation _Platform-Computation.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\justi\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\Raquel_HRD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC0CC056-9AC3-41C2-8E16-D14854ADAFFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D965BF7F-916C-46BF-9BE6-8EB0E3B7EFA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{22A5745B-9E59-4E91-9FA4-3C7DB1ABBFEE}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="23">
   <si>
     <t>Rating Scale</t>
   </si>
@@ -101,35 +101,20 @@
     <t>Final Department State (after all employees complete)</t>
   </si>
   <si>
-    <t>Eduardo Aquino</t>
-  </si>
-  <si>
-    <t>Leonora Gomez</t>
-  </si>
-  <si>
-    <t>Ronald Lopez</t>
-  </si>
-  <si>
-    <t>Christopher Tolentino</t>
-  </si>
-  <si>
-    <t>VP for Acquired Properties</t>
-  </si>
-  <si>
-    <t>AP Staff I</t>
-  </si>
-  <si>
-    <t>AP Supervisor I</t>
-  </si>
-  <si>
-    <t>AP Manager I</t>
+    <t>Elena Delgado</t>
+  </si>
+  <si>
+    <t>HR Supervisor</t>
+  </si>
+  <si>
+    <t>HR Manager</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -168,6 +153,13 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF1A2E06"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="7">
@@ -326,9 +318,6 @@
     <xf numFmtId="2" fontId="0" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -336,6 +325,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="2" fontId="4" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -728,121 +720,79 @@
       <c r="G2" s="1"/>
       <c r="H2" s="1"/>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A3" s="15" t="s">
+    <row r="3" spans="1:8" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A3" s="18" t="s">
         <v>20</v>
       </c>
-      <c r="B3" s="17" t="s">
-        <v>24</v>
-      </c>
-      <c r="C3" s="16">
-        <v>3.8</v>
-      </c>
-      <c r="D3" s="16">
-        <v>2.5</v>
+      <c r="B3" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="C3" s="15">
+        <v>4</v>
+      </c>
+      <c r="D3" s="15">
+        <v>4</v>
       </c>
       <c r="E3" s="7">
         <f>C3*$E$1+D3*$H$1</f>
-        <v>3.54</v>
+        <v>4</v>
       </c>
       <c r="F3" s="6" t="str">
         <f>IF(E3&gt;=3.6,"Outstanding",IF(E3&gt;=2.6,"Exceeds Expectations",IF(E3&gt;=2,"Meets Expectations","Needs Improvement")))</f>
-        <v>Exceeds Expectations</v>
+        <v>Outstanding</v>
       </c>
       <c r="G3" s="1"/>
       <c r="H3" s="1"/>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A4" s="15" t="s">
+    <row r="4" spans="1:8" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A4" s="18" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="B4" s="17" t="s">
-        <v>25</v>
-      </c>
-      <c r="C4" s="18">
-        <v>4</v>
-      </c>
-      <c r="D4" s="16">
-        <v>2.38</v>
+      <c r="C4" s="17">
+        <v>1</v>
+      </c>
+      <c r="D4" s="15">
+        <v>1</v>
       </c>
       <c r="E4" s="7">
         <f>C4*$E$1+D4*$H$1</f>
-        <v>3.6760000000000002</v>
+        <v>1</v>
       </c>
       <c r="F4" s="6" t="str">
         <f t="shared" ref="F4:F7" si="0">IF(E4&gt;=3.6,"Outstanding",IF(E4&gt;=2.6,"Exceeds Expectations",IF(E4&gt;=2,"Meets Expectations","Needs Improvement")))</f>
-        <v>Outstanding</v>
+        <v>Needs Improvement</v>
       </c>
       <c r="G4" s="1"/>
       <c r="H4" s="1"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" s="15" t="s">
-        <v>10</v>
-      </c>
-      <c r="B5" s="17" t="s">
-        <v>26</v>
-      </c>
-      <c r="C5" s="18">
-        <v>4</v>
-      </c>
-      <c r="D5" s="16">
-        <v>3.13</v>
-      </c>
-      <c r="E5" s="7">
-        <f t="shared" ref="E5:E7" si="1">C5*$E$1+D5*$H$1</f>
-        <v>3.8260000000000001</v>
-      </c>
-      <c r="F5" s="6" t="str">
-        <f t="shared" si="0"/>
-        <v>Outstanding</v>
-      </c>
+      <c r="A5" s="6"/>
+      <c r="B5" s="16"/>
+      <c r="C5" s="17"/>
+      <c r="D5" s="15"/>
+      <c r="E5" s="7"/>
+      <c r="F5" s="6"/>
       <c r="G5" s="1"/>
       <c r="H5" s="1"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A6" s="16" t="s">
-        <v>22</v>
-      </c>
-      <c r="B6" s="17" t="s">
-        <v>26</v>
-      </c>
-      <c r="C6" s="18">
-        <v>4</v>
-      </c>
-      <c r="D6" s="16">
-        <v>2.63</v>
-      </c>
-      <c r="E6" s="7">
-        <f t="shared" si="1"/>
-        <v>3.726</v>
-      </c>
-      <c r="F6" s="6" t="str">
-        <f t="shared" si="0"/>
-        <v>Outstanding</v>
-      </c>
+      <c r="A6" s="15"/>
+      <c r="B6" s="16"/>
+      <c r="C6" s="17"/>
+      <c r="D6" s="15"/>
+      <c r="E6" s="7"/>
+      <c r="F6" s="6"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A7" s="16" t="s">
-        <v>23</v>
-      </c>
-      <c r="B7" s="17" t="s">
-        <v>27</v>
-      </c>
-      <c r="C7" s="18">
-        <v>4</v>
-      </c>
-      <c r="D7" s="18">
-        <v>4</v>
-      </c>
-      <c r="E7" s="7">
-        <f t="shared" si="1"/>
-        <v>4</v>
-      </c>
-      <c r="F7" s="6" t="str">
-        <f t="shared" si="0"/>
-        <v>Outstanding</v>
-      </c>
+      <c r="A7" s="15"/>
+      <c r="B7" s="16"/>
+      <c r="C7" s="17"/>
+      <c r="D7" s="17"/>
+      <c r="E7" s="7"/>
+      <c r="F7" s="6"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
@@ -866,11 +816,11 @@
       </c>
       <c r="B11" s="9">
         <f>COUNTA(A3:A7)</f>
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C11" s="10">
         <f>AVERAGE(D3:D7)</f>
-        <v>2.9279999999999999</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
@@ -908,23 +858,23 @@
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="9" t="str">
         <f>A3</f>
-        <v>Eduardo Aquino</v>
+        <v>Elena Delgado</v>
       </c>
       <c r="B16" s="10">
-        <f>C3</f>
-        <v>3.8</v>
+        <f t="shared" ref="B16:C20" si="1">C3</f>
+        <v>4</v>
       </c>
       <c r="C16" s="10">
-        <f>D3</f>
-        <v>2.5</v>
+        <f t="shared" si="1"/>
+        <v>4</v>
       </c>
       <c r="D16" s="10">
         <f>C11</f>
-        <v>2.9279999999999999</v>
+        <v>2.5</v>
       </c>
       <c r="E16" s="14">
         <f>B16*$E$1+D16*$H$1</f>
-        <v>3.6255999999999999</v>
+        <v>3.7</v>
       </c>
       <c r="F16" s="9" t="str">
         <f>IF(E16&gt;=3.6,"Outstanding",IF(E16&gt;=2.6,"Exceeds Expectations",IF(E16&gt;=2,"Meets Expectations","Needs Improvement")))</f>
@@ -934,106 +884,52 @@
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="9" t="str">
         <f>A4</f>
-        <v>Leonora Gomez</v>
+        <v>Patricia Gomez</v>
       </c>
       <c r="B17" s="10">
-        <f>C4</f>
-        <v>4</v>
+        <f t="shared" si="1"/>
+        <v>1</v>
       </c>
       <c r="C17" s="10">
-        <f>D4</f>
-        <v>2.38</v>
+        <f t="shared" si="1"/>
+        <v>1</v>
       </c>
       <c r="D17" s="10">
         <f>C11</f>
-        <v>2.9279999999999999</v>
+        <v>2.5</v>
       </c>
       <c r="E17" s="14">
         <f t="shared" ref="E17:E20" si="2">B17*$E$1+D17*$H$1</f>
-        <v>3.7856000000000001</v>
+        <v>1.3</v>
       </c>
       <c r="F17" s="9" t="str">
         <f t="shared" ref="F17:F20" si="3">IF(E17&gt;=3.6,"Outstanding",IF(E17&gt;=2.6,"Exceeds Expectations",IF(E17&gt;=2,"Meets Expectations","Needs Improvement")))</f>
-        <v>Outstanding</v>
+        <v>Needs Improvement</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A18" s="9" t="str">
-        <f>A5</f>
-        <v>Patricia Gomez</v>
-      </c>
-      <c r="B18" s="10">
-        <f>C5</f>
-        <v>4</v>
-      </c>
-      <c r="C18" s="10">
-        <f>D5</f>
-        <v>3.13</v>
-      </c>
-      <c r="D18" s="10">
-        <f>C11</f>
-        <v>2.9279999999999999</v>
-      </c>
-      <c r="E18" s="14">
-        <f t="shared" si="2"/>
-        <v>3.7856000000000001</v>
-      </c>
-      <c r="F18" s="9" t="str">
-        <f t="shared" si="3"/>
-        <v>Outstanding</v>
-      </c>
+      <c r="A18" s="9"/>
+      <c r="B18" s="10"/>
+      <c r="C18" s="10"/>
+      <c r="D18" s="10"/>
+      <c r="E18" s="14"/>
+      <c r="F18" s="9"/>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A19" s="9" t="str">
-        <f>A6</f>
-        <v>Ronald Lopez</v>
-      </c>
-      <c r="B19" s="10">
-        <f>C6</f>
-        <v>4</v>
-      </c>
-      <c r="C19" s="10">
-        <f>D6</f>
-        <v>2.63</v>
-      </c>
-      <c r="D19" s="10">
-        <f>C11</f>
-        <v>2.9279999999999999</v>
-      </c>
-      <c r="E19" s="14">
-        <f t="shared" si="2"/>
-        <v>3.7856000000000001</v>
-      </c>
-      <c r="F19" s="9" t="str">
-        <f t="shared" si="3"/>
-        <v>Outstanding</v>
-      </c>
+      <c r="A19" s="9"/>
+      <c r="B19" s="10"/>
+      <c r="C19" s="10"/>
+      <c r="D19" s="10"/>
+      <c r="E19" s="14"/>
+      <c r="F19" s="9"/>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A20" s="9" t="str">
-        <f>A7</f>
-        <v>Christopher Tolentino</v>
-      </c>
-      <c r="B20" s="10">
-        <f>C7</f>
-        <v>4</v>
-      </c>
-      <c r="C20" s="10">
-        <f>D7</f>
-        <v>4</v>
-      </c>
-      <c r="D20" s="10">
-        <f>C11</f>
-        <v>2.9279999999999999</v>
-      </c>
-      <c r="E20" s="14">
-        <f t="shared" si="2"/>
-        <v>3.7856000000000001</v>
-      </c>
-      <c r="F20" s="9" t="str">
-        <f t="shared" si="3"/>
-        <v>Outstanding</v>
-      </c>
+      <c r="A20" s="9"/>
+      <c r="B20" s="10"/>
+      <c r="C20" s="10"/>
+      <c r="D20" s="10"/>
+      <c r="E20" s="14"/>
+      <c r="F20" s="9"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Update workforce analytics computation workbook
</commit_message>
<xml_diff>
--- a/Raquel_Pawnshop_HR_Workforce_Analytics_&_Evaluation _Platform-Computation.xlsx
+++ b/Raquel_Pawnshop_HR_Workforce_Analytics_&_Evaluation _Platform-Computation.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\Raquel_HRD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A35C41F6-BBC8-40AA-8164-7B8E413B4F79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C56D877B-2B3A-4A44-AAD8-347B0CFB3CCE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{22A5745B-9E59-4E91-9FA4-3C7DB1ABBFEE}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="28">
   <si>
     <t>Rating Scale</t>
   </si>
@@ -71,9 +71,6 @@
     <t>Status</t>
   </si>
   <si>
-    <t>Patricia Gomez</t>
-  </si>
-  <si>
     <t>Department</t>
   </si>
   <si>
@@ -101,19 +98,31 @@
     <t>Final Department State (after all employees complete)</t>
   </si>
   <si>
-    <t>Elena Delgado</t>
-  </si>
-  <si>
-    <t>HR Supervisor</t>
-  </si>
-  <si>
-    <t>HR Manager</t>
-  </si>
-  <si>
-    <t>Miguel Torres</t>
-  </si>
-  <si>
-    <t>HR Staff</t>
+    <t>elena</t>
+  </si>
+  <si>
+    <t>patricia</t>
+  </si>
+  <si>
+    <t>miguel</t>
+  </si>
+  <si>
+    <t>james</t>
+  </si>
+  <si>
+    <t>fred</t>
+  </si>
+  <si>
+    <t>hr manager</t>
+  </si>
+  <si>
+    <t>hr supervisor</t>
+  </si>
+  <si>
+    <t>hr staff</t>
+  </si>
+  <si>
+    <t>hr staff II</t>
   </si>
 </sst>
 </file>
@@ -162,8 +171,8 @@
     </font>
     <font>
       <b/>
-      <sz val="11"/>
-      <color rgb="FF1A2E06"/>
+      <sz val="10"/>
+      <color rgb="FF0F172A"/>
       <name val="Segoe UI"/>
       <family val="2"/>
     </font>
@@ -726,22 +735,22 @@
       <c r="G2" s="1"/>
       <c r="H2" s="1"/>
     </row>
-    <row r="3" spans="1:8" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="18" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B3" s="16" t="s">
-        <v>22</v>
-      </c>
-      <c r="C3" s="15">
+        <v>24</v>
+      </c>
+      <c r="C3" s="17">
         <v>4</v>
       </c>
-      <c r="D3" s="15">
-        <v>4</v>
+      <c r="D3" s="17">
+        <v>3.88</v>
       </c>
       <c r="E3" s="7">
         <f>C3*$E$1+D3*$H$1</f>
-        <v>4</v>
+        <v>3.976</v>
       </c>
       <c r="F3" s="6" t="str">
         <f>IF(E3&gt;=3.6,"Outstanding",IF(E3&gt;=2.6,"Exceeds Expectations",IF(E3&gt;=2,"Meets Expectations","Needs Improvement")))</f>
@@ -750,97 +759,119 @@
       <c r="G3" s="1"/>
       <c r="H3" s="1"/>
     </row>
-    <row r="4" spans="1:8" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="18" t="s">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="B4" s="16" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="C4" s="17">
-        <v>1</v>
-      </c>
-      <c r="D4" s="15">
-        <v>1</v>
+        <v>3.4</v>
+      </c>
+      <c r="D4" s="17">
+        <v>3.75</v>
       </c>
       <c r="E4" s="7">
         <f>C4*$E$1+D4*$H$1</f>
-        <v>1</v>
+        <v>3.47</v>
       </c>
       <c r="F4" s="6" t="str">
         <f t="shared" ref="F4:F7" si="0">IF(E4&gt;=3.6,"Outstanding",IF(E4&gt;=2.6,"Exceeds Expectations",IF(E4&gt;=2,"Meets Expectations","Needs Improvement")))</f>
-        <v>Needs Improvement</v>
+        <v>Exceeds Expectations</v>
       </c>
       <c r="G4" s="1"/>
       <c r="H4" s="1"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" s="6" t="s">
-        <v>23</v>
+      <c r="A5" s="18" t="s">
+        <v>21</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C5" s="17">
-        <v>2</v>
-      </c>
-      <c r="D5" s="15">
         <v>3</v>
+      </c>
+      <c r="D5" s="17">
+        <v>3.75</v>
       </c>
       <c r="E5" s="7">
         <f>C5*$E$1+D5*$H$1</f>
-        <v>2.2000000000000002</v>
+        <v>3.1500000000000004</v>
       </c>
       <c r="F5" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>Meets Expectations</v>
+        <v>Exceeds Expectations</v>
       </c>
       <c r="G5" s="1"/>
       <c r="H5" s="1"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A6" s="15"/>
-      <c r="B6" s="16"/>
-      <c r="C6" s="17"/>
-      <c r="D6" s="15"/>
-      <c r="E6" s="7"/>
-      <c r="F6" s="6"/>
+      <c r="A6" s="18" t="s">
+        <v>22</v>
+      </c>
+      <c r="B6" s="16" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" s="17">
+        <v>4</v>
+      </c>
+      <c r="D6" s="15">
+        <v>3.5</v>
+      </c>
+      <c r="E6" s="7">
+        <f>C6*$E$1+D6*$H$1</f>
+        <v>3.9000000000000004</v>
+      </c>
+      <c r="F6" s="6" t="str">
+        <f t="shared" si="0"/>
+        <v>Outstanding</v>
+      </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A7" s="15"/>
+      <c r="A7" s="18" t="s">
+        <v>23</v>
+      </c>
       <c r="B7" s="16"/>
       <c r="C7" s="17"/>
       <c r="D7" s="17"/>
-      <c r="E7" s="7"/>
-      <c r="F7" s="6"/>
+      <c r="E7" s="7">
+        <f t="shared" ref="E7" si="1">C7*$E$1+D7*$H$1</f>
+        <v>0</v>
+      </c>
+      <c r="F7" s="6" t="str">
+        <f t="shared" si="0"/>
+        <v>Needs Improvement</v>
+      </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B10" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="B10" s="8" t="s">
+      <c r="C10" s="8" t="s">
         <v>12</v>
-      </c>
-      <c r="C10" s="8" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B11" s="9">
         <f>COUNTA(A3:A7)</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C11" s="10">
         <f>AVERAGE(D3:D7)</f>
-        <v>2.6666666666666665</v>
+        <v>3.7199999999999998</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
@@ -850,7 +881,7 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B13" s="4"/>
       <c r="C13" s="5"/>
@@ -860,41 +891,41 @@
         <v>4</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C15" s="13" t="s">
         <v>7</v>
       </c>
       <c r="D15" s="13" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E15" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="F15" s="13" t="s">
         <v>17</v>
-      </c>
-      <c r="F15" s="13" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="9" t="str">
         <f>A3</f>
-        <v>Elena Delgado</v>
+        <v>elena</v>
       </c>
       <c r="B16" s="10">
-        <f t="shared" ref="B16:C20" si="1">C3</f>
+        <f t="shared" ref="B16:C19" si="2">C3</f>
         <v>4</v>
       </c>
       <c r="C16" s="10">
-        <f t="shared" si="1"/>
-        <v>4</v>
+        <f t="shared" si="2"/>
+        <v>3.88</v>
       </c>
       <c r="D16" s="10">
         <f>$C$11</f>
-        <v>2.6666666666666665</v>
+        <v>3.7199999999999998</v>
       </c>
       <c r="E16" s="14">
         <f>B16*$E$1+D16*$H$1</f>
-        <v>3.7333333333333334</v>
+        <v>3.944</v>
       </c>
       <c r="F16" s="9" t="str">
         <f>IF(E16&gt;=3.6,"Outstanding",IF(E16&gt;=2.6,"Exceeds Expectations",IF(E16&gt;=2,"Meets Expectations","Needs Improvement")))</f>
@@ -904,72 +935,109 @@
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="9" t="str">
         <f>A4</f>
-        <v>Patricia Gomez</v>
+        <v>patricia</v>
       </c>
       <c r="B17" s="10">
-        <f t="shared" si="1"/>
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>3.4</v>
       </c>
       <c r="C17" s="10">
-        <f t="shared" si="1"/>
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>3.75</v>
       </c>
       <c r="D17" s="10">
-        <f t="shared" ref="D17:D18" si="2">$C$11</f>
-        <v>2.6666666666666665</v>
+        <f t="shared" ref="D17:D19" si="3">$C$11</f>
+        <v>3.7199999999999998</v>
       </c>
       <c r="E17" s="14">
-        <f t="shared" ref="E17:E20" si="3">B17*$E$1+D17*$H$1</f>
-        <v>1.3333333333333335</v>
+        <f t="shared" ref="E17" si="4">B17*$E$1+D17*$H$1</f>
+        <v>3.4640000000000004</v>
       </c>
       <c r="F17" s="9" t="str">
-        <f t="shared" ref="F17:F20" si="4">IF(E17&gt;=3.6,"Outstanding",IF(E17&gt;=2.6,"Exceeds Expectations",IF(E17&gt;=2,"Meets Expectations","Needs Improvement")))</f>
-        <v>Needs Improvement</v>
+        <f t="shared" ref="F17" si="5">IF(E17&gt;=3.6,"Outstanding",IF(E17&gt;=2.6,"Exceeds Expectations",IF(E17&gt;=2,"Meets Expectations","Needs Improvement")))</f>
+        <v>Exceeds Expectations</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="9" t="str">
         <f>A5</f>
-        <v>Miguel Torres</v>
+        <v>miguel</v>
       </c>
       <c r="B18" s="10">
-        <f t="shared" si="1"/>
-        <v>2</v>
+        <f t="shared" si="2"/>
+        <v>3</v>
       </c>
       <c r="C18" s="10">
-        <f t="shared" si="1"/>
-        <v>3</v>
+        <f t="shared" si="2"/>
+        <v>3.75</v>
       </c>
       <c r="D18" s="10">
+        <f t="shared" si="3"/>
+        <v>3.7199999999999998</v>
+      </c>
+      <c r="E18" s="14">
+        <f t="shared" ref="E18:E20" si="6">B18*$E$1+D18*$H$1</f>
+        <v>3.1440000000000001</v>
+      </c>
+      <c r="F18" s="9" t="str">
+        <f t="shared" ref="F18:F20" si="7">IF(E18&gt;=3.6,"Outstanding",IF(E18&gt;=2.6,"Exceeds Expectations",IF(E18&gt;=2,"Meets Expectations","Needs Improvement")))</f>
+        <v>Exceeds Expectations</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" s="9" t="str">
+        <f>A6</f>
+        <v>james</v>
+      </c>
+      <c r="B19" s="10">
         <f t="shared" si="2"/>
-        <v>2.6666666666666665</v>
-      </c>
-      <c r="E18" s="14">
-        <f t="shared" ref="E18" si="5">B18*$E$1+D18*$H$1</f>
-        <v>2.1333333333333333</v>
-      </c>
-      <c r="F18" s="9" t="str">
-        <f t="shared" ref="F18" si="6">IF(E18&gt;=3.6,"Outstanding",IF(E18&gt;=2.6,"Exceeds Expectations",IF(E18&gt;=2,"Meets Expectations","Needs Improvement")))</f>
-        <v>Meets Expectations</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A19" s="9"/>
-      <c r="B19" s="10"/>
-      <c r="C19" s="10"/>
-      <c r="D19" s="10"/>
-      <c r="E19" s="14"/>
-      <c r="F19" s="9"/>
+        <v>4</v>
+      </c>
+      <c r="C19" s="10">
+        <f t="shared" si="2"/>
+        <v>3.5</v>
+      </c>
+      <c r="D19" s="10">
+        <f t="shared" si="3"/>
+        <v>3.7199999999999998</v>
+      </c>
+      <c r="E19" s="14">
+        <f t="shared" si="6"/>
+        <v>3.944</v>
+      </c>
+      <c r="F19" s="9" t="str">
+        <f t="shared" si="7"/>
+        <v>Outstanding</v>
+      </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A20" s="9"/>
-      <c r="B20" s="10"/>
-      <c r="C20" s="10"/>
-      <c r="D20" s="10"/>
-      <c r="E20" s="14"/>
-      <c r="F20" s="9"/>
+      <c r="A20" s="9" t="str">
+        <f>A7</f>
+        <v>fred</v>
+      </c>
+      <c r="B20" s="10">
+        <f>C7</f>
+        <v>0</v>
+      </c>
+      <c r="C20" s="10">
+        <f>D7</f>
+        <v>0</v>
+      </c>
+      <c r="D20" s="10">
+        <f>C11</f>
+        <v>3.7199999999999998</v>
+      </c>
+      <c r="E20" s="14">
+        <f t="shared" si="6"/>
+        <v>0.74399999999999999</v>
+      </c>
+      <c r="F20" s="9" t="str">
+        <f t="shared" si="7"/>
+        <v>Needs Improvement</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
new Performance Evaluation rebrand
</commit_message>
<xml_diff>
--- a/Raquel_Pawnshop_HR_Workforce_Analytics_&_Evaluation _Platform-Computation.xlsx
+++ b/Raquel_Pawnshop_HR_Workforce_Analytics_&_Evaluation _Platform-Computation.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\Raquel_HRD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E0605A8-B670-457B-9EE3-FE1C7C0F2054}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BDD72C4-C495-4FA8-841E-55081E81150B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{22A5745B-9E59-4E91-9FA4-3C7DB1ABBFEE}"/>
   </bookViews>
@@ -955,56 +955,20 @@
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A19" s="9">
-        <f>A6</f>
-        <v>0</v>
-      </c>
-      <c r="B19" s="10">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="C19" s="10">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="D19" s="10">
-        <f t="shared" si="2"/>
-        <v>3.0033333333333334</v>
-      </c>
-      <c r="E19" s="14">
-        <f t="shared" si="5"/>
-        <v>0.60066666666666668</v>
-      </c>
-      <c r="F19" s="9" t="str">
-        <f t="shared" si="6"/>
-        <v>Needs Improvement</v>
-      </c>
+      <c r="A19" s="9"/>
+      <c r="B19" s="10"/>
+      <c r="C19" s="10"/>
+      <c r="D19" s="10"/>
+      <c r="E19" s="14"/>
+      <c r="F19" s="9"/>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A20" s="9">
-        <f>A7</f>
-        <v>0</v>
-      </c>
-      <c r="B20" s="10">
-        <f>C7</f>
-        <v>0</v>
-      </c>
-      <c r="C20" s="10">
-        <f>D7</f>
-        <v>0</v>
-      </c>
-      <c r="D20" s="10">
-        <f>C11</f>
-        <v>3.0033333333333334</v>
-      </c>
-      <c r="E20" s="14">
-        <f t="shared" si="5"/>
-        <v>0.60066666666666668</v>
-      </c>
-      <c r="F20" s="9" t="str">
-        <f t="shared" si="6"/>
-        <v>Needs Improvement</v>
-      </c>
+      <c r="A20" s="9"/>
+      <c r="B20" s="10"/>
+      <c r="C20" s="10"/>
+      <c r="D20" s="10"/>
+      <c r="E20" s="14"/>
+      <c r="F20" s="9"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Implement probationary evaluation workflow and template controls
Route probationary evaluations through department review and HR final approval, retain the employee's original self-rating signature, and present score comparisons and signatures in evaluation details. Keep ongoing reviews out of Evaluation History.

Restrict template browsing to the viewer's department while preserving HR cross-department visibility. Allow department managers and supervisors to manage one another's templates within their department, with existing safeguards for templates already in use.

Update probationary employee setup, portal access, supporting schema, implementation notes, and workflow regression coverage.
</commit_message>
<xml_diff>
--- a/Raquel_Pawnshop_HR_Workforce_Analytics_&_Evaluation _Platform-Computation.xlsx
+++ b/Raquel_Pawnshop_HR_Workforce_Analytics_&_Evaluation _Platform-Computation.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\Raquel_HRD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{304962BB-8DA2-4ADD-930A-E334EA290764}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8434E25F-FA25-4B20-88F8-8E8155F88F4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{22A5745B-9E59-4E91-9FA4-3C7DB1ABBFEE}"/>
   </bookViews>
@@ -778,14 +778,14 @@
         <v>18</v>
       </c>
       <c r="C3" s="17">
-        <v>2.65</v>
+        <v>2.97</v>
       </c>
       <c r="D3" s="17">
-        <v>2.88</v>
+        <v>2.63</v>
       </c>
       <c r="E3" s="7">
         <f>C3*$E$1+D3*$G$1</f>
-        <v>2.6960000000000002</v>
+        <v>2.9020000000000001</v>
       </c>
       <c r="F3" s="6" t="str">
         <f>IF(E3&gt;=3.6,"Outstanding",
@@ -804,20 +804,20 @@
         <v>19</v>
       </c>
       <c r="C4" s="17">
-        <v>2.8</v>
+        <v>2.0499999999999998</v>
       </c>
       <c r="D4" s="17">
-        <v>3</v>
+        <v>2.13</v>
       </c>
       <c r="E4" s="7">
         <f>C4*$E$1+D4*$G$1</f>
-        <v>2.84</v>
+        <v>2.0659999999999998</v>
       </c>
       <c r="F4" s="6" t="str">
         <f t="shared" ref="F4:F5" si="0">IF(E4&gt;=3.6,"Outstanding",
  IF(E4&gt;=2.6,"Exceeds Expectations",
  IF(E4&gt;=2,"Meets Expectations","Needs Improvement")))</f>
-        <v>Exceeds Expectations</v>
+        <v>Meets Expectations</v>
       </c>
       <c r="G4" s="1"/>
       <c r="H4" s="1"/>
@@ -829,19 +829,15 @@
       <c r="B5" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="C5" s="17">
-        <v>2.88</v>
-      </c>
-      <c r="D5" s="17">
-        <v>3.13</v>
-      </c>
+      <c r="C5" s="17"/>
+      <c r="D5" s="17"/>
       <c r="E5" s="7">
         <f>C5*$E$1+D5*$G$1</f>
-        <v>2.9299999999999997</v>
+        <v>0</v>
       </c>
       <c r="F5" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>Exceeds Expectations</v>
+        <v>Needs Improvement</v>
       </c>
       <c r="G5" s="1"/>
       <c r="H5" s="1"/>
@@ -888,7 +884,7 @@
       </c>
       <c r="C11" s="10">
         <f>AVERAGE(D3:D7)</f>
-        <v>3.0033333333333334</v>
+        <v>2.38</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
@@ -932,19 +928,19 @@
       </c>
       <c r="B16" s="10">
         <f t="shared" ref="B16:C18" si="1">C3</f>
-        <v>2.65</v>
+        <v>2.97</v>
       </c>
       <c r="C16" s="10">
         <f t="shared" si="1"/>
-        <v>2.88</v>
+        <v>2.63</v>
       </c>
       <c r="D16" s="10">
         <f>$C$11</f>
-        <v>3.0033333333333334</v>
+        <v>2.38</v>
       </c>
       <c r="E16" s="14">
         <f>B16*$E$1+D16*$G$1</f>
-        <v>2.7206666666666668</v>
+        <v>2.8520000000000003</v>
       </c>
       <c r="F16" s="9" t="str">
         <f>IF(E16&gt;=3.6,"Outstanding",
@@ -960,25 +956,25 @@
       </c>
       <c r="B17" s="10">
         <f t="shared" si="1"/>
-        <v>2.8</v>
+        <v>2.0499999999999998</v>
       </c>
       <c r="C17" s="10">
         <f t="shared" si="1"/>
-        <v>3</v>
+        <v>2.13</v>
       </c>
       <c r="D17" s="10">
         <f t="shared" ref="D17:D18" si="2">$C$11</f>
-        <v>3.0033333333333334</v>
+        <v>2.38</v>
       </c>
       <c r="E17" s="14">
         <f>B17*$E$1+D17*$G$1</f>
-        <v>2.8406666666666665</v>
+        <v>2.1159999999999997</v>
       </c>
       <c r="F17" s="9" t="str">
         <f t="shared" ref="F17:F18" si="3">IF(E17&gt;=3.6,"Outstanding",
  IF(E17&gt;=2.6,"Exceeds Expectations",
  IF(E17&gt;=2,"Meets Expectations","Needs Improvement")))</f>
-        <v>Exceeds Expectations</v>
+        <v>Meets Expectations</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
@@ -988,23 +984,23 @@
       </c>
       <c r="B18" s="10">
         <f t="shared" si="1"/>
-        <v>2.88</v>
+        <v>0</v>
       </c>
       <c r="C18" s="10">
         <f t="shared" si="1"/>
-        <v>3.13</v>
+        <v>0</v>
       </c>
       <c r="D18" s="10">
         <f t="shared" si="2"/>
-        <v>3.0033333333333334</v>
+        <v>2.38</v>
       </c>
       <c r="E18" s="14">
         <f>B18*$E$1+D18*$G$1</f>
-        <v>2.9046666666666665</v>
+        <v>0.47599999999999998</v>
       </c>
       <c r="F18" s="9" t="str">
         <f t="shared" si="3"/>
-        <v>Exceeds Expectations</v>
+        <v>Needs Improvement</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Enhance probationary evaluation process by adding eligibility checks and finalization logic, updating relevant employee status and notifications
</commit_message>
<xml_diff>
--- a/Raquel_Pawnshop_HR_Workforce_Analytics_&_Evaluation _Platform-Computation.xlsx
+++ b/Raquel_Pawnshop_HR_Workforce_Analytics_&_Evaluation _Platform-Computation.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\Raquel_HRD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8434E25F-FA25-4B20-88F8-8E8155F88F4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{642FECBF-AB68-40BB-A10A-A0182D274CE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{22A5745B-9E59-4E91-9FA4-3C7DB1ABBFEE}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{22A5745B-9E59-4E91-9FA4-3C7DB1ABBFEE}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -79,7 +79,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="19">
   <si>
     <t>Rating Scale</t>
   </si>
@@ -126,24 +126,6 @@
     <t>Final Department State (after all employees complete)</t>
   </si>
   <si>
-    <t>elena</t>
-  </si>
-  <si>
-    <t>patricia</t>
-  </si>
-  <si>
-    <t>miguel</t>
-  </si>
-  <si>
-    <t>hr manager</t>
-  </si>
-  <si>
-    <t>hr supervisor</t>
-  </si>
-  <si>
-    <t>hr staff</t>
-  </si>
-  <si>
     <t>Self Core Values</t>
   </si>
   <si>
@@ -151,13 +133,16 @@
   </si>
   <si>
     <t>Score</t>
+  </si>
+  <si>
+    <t>liana</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -716,18 +701,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A83BB1C1-F953-4E33-A206-594A5C40587D}">
   <dimension ref="A1:H20"/>
-  <sheetFormatPr defaultColWidth="26" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="26" defaultRowHeight="14"/>
   <cols>
-    <col min="1" max="1" width="52.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="20.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.5703125" customWidth="1"/>
+    <col min="1" max="1" width="52.1640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.75" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="20.4140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.58203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.83203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.58203125" customWidth="1"/>
     <col min="8" max="8" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8">
       <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
@@ -748,7 +733,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" ht="14.5">
       <c r="A2" s="11" t="s">
         <v>4</v>
       </c>
@@ -756,13 +741,13 @@
         <v>5</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D2" s="11" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="E2" s="11" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="F2" s="11" t="s">
         <v>6</v>
@@ -770,65 +755,47 @@
       <c r="G2" s="1"/>
       <c r="H2" s="1"/>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" ht="16">
       <c r="A3" s="18" t="s">
-        <v>15</v>
-      </c>
-      <c r="B3" s="16" t="s">
         <v>18</v>
       </c>
-      <c r="C3" s="17">
-        <v>2.97</v>
-      </c>
-      <c r="D3" s="17">
-        <v>2.63</v>
-      </c>
+      <c r="B3" s="16"/>
+      <c r="C3" s="17"/>
+      <c r="D3" s="17"/>
       <c r="E3" s="7">
         <f>C3*$E$1+D3*$G$1</f>
-        <v>2.9020000000000001</v>
+        <v>0</v>
       </c>
       <c r="F3" s="6" t="str">
         <f>IF(E3&gt;=3.6,"Outstanding",
  IF(E3&gt;=2.6,"Exceeds Expectations",
  IF(E3&gt;=2,"Meets Expectations","Needs Improvement")))</f>
-        <v>Exceeds Expectations</v>
+        <v>Needs Improvement</v>
       </c>
       <c r="G3" s="1"/>
       <c r="H3" s="1"/>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A4" s="18" t="s">
-        <v>16</v>
-      </c>
-      <c r="B4" s="16" t="s">
-        <v>19</v>
-      </c>
-      <c r="C4" s="17">
-        <v>2.0499999999999998</v>
-      </c>
-      <c r="D4" s="17">
-        <v>2.13</v>
-      </c>
+    <row r="4" spans="1:8" ht="16">
+      <c r="A4" s="18"/>
+      <c r="B4" s="16"/>
+      <c r="C4" s="17"/>
+      <c r="D4" s="17"/>
       <c r="E4" s="7">
         <f>C4*$E$1+D4*$G$1</f>
-        <v>2.0659999999999998</v>
+        <v>0</v>
       </c>
       <c r="F4" s="6" t="str">
         <f t="shared" ref="F4:F5" si="0">IF(E4&gt;=3.6,"Outstanding",
  IF(E4&gt;=2.6,"Exceeds Expectations",
  IF(E4&gt;=2,"Meets Expectations","Needs Improvement")))</f>
-        <v>Meets Expectations</v>
+        <v>Needs Improvement</v>
       </c>
       <c r="G4" s="1"/>
       <c r="H4" s="1"/>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" s="18" t="s">
-        <v>17</v>
-      </c>
-      <c r="B5" s="16" t="s">
-        <v>20</v>
-      </c>
+    <row r="5" spans="1:8" ht="16">
+      <c r="A5" s="18"/>
+      <c r="B5" s="16"/>
       <c r="C5" s="17"/>
       <c r="D5" s="17"/>
       <c r="E5" s="7">
@@ -842,7 +809,7 @@
       <c r="G5" s="1"/>
       <c r="H5" s="1"/>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" ht="16">
       <c r="A6" s="18"/>
       <c r="B6" s="16"/>
       <c r="C6" s="17"/>
@@ -850,7 +817,7 @@
       <c r="E6" s="6"/>
       <c r="F6" s="19"/>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" ht="16">
       <c r="A7" s="18"/>
       <c r="B7" s="16"/>
       <c r="C7" s="17"/>
@@ -858,12 +825,12 @@
       <c r="E7" s="6"/>
       <c r="F7" s="19"/>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8">
       <c r="A8" s="2" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" ht="14.5">
       <c r="A10" s="8" t="s">
         <v>7</v>
       </c>
@@ -874,32 +841,32 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8">
       <c r="A11" s="9" t="s">
         <v>10</v>
       </c>
       <c r="B11" s="9">
         <f>COUNTA(A3:A7)</f>
-        <v>3</v>
-      </c>
-      <c r="C11" s="10">
+        <v>1</v>
+      </c>
+      <c r="C11" s="10" t="e">
         <f>AVERAGE(D3:D7)</f>
-        <v>2.38</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8">
       <c r="A12" s="1"/>
       <c r="B12" s="1"/>
       <c r="C12" s="1"/>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8" ht="14.5">
       <c r="A13" s="3" t="s">
         <v>11</v>
       </c>
       <c r="B13" s="4"/>
       <c r="C13" s="5"/>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:8" ht="14.5">
       <c r="A15" s="13" t="s">
         <v>4</v>
       </c>
@@ -921,66 +888,66 @@
         <v>13</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:8">
       <c r="A16" s="9" t="str">
         <f>A3</f>
-        <v>elena</v>
+        <v>liana</v>
       </c>
       <c r="B16" s="10">
         <f t="shared" ref="B16:C18" si="1">C3</f>
-        <v>2.97</v>
+        <v>0</v>
       </c>
       <c r="C16" s="10">
         <f t="shared" si="1"/>
-        <v>2.63</v>
-      </c>
-      <c r="D16" s="10">
+        <v>0</v>
+      </c>
+      <c r="D16" s="10" t="e">
         <f>$C$11</f>
-        <v>2.38</v>
-      </c>
-      <c r="E16" s="14">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="E16" s="14" t="e">
         <f>B16*$E$1+D16*$G$1</f>
-        <v>2.8520000000000003</v>
-      </c>
-      <c r="F16" s="9" t="str">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="F16" s="9" t="e">
         <f>IF(E16&gt;=3.6,"Outstanding",
  IF(E16&gt;=2.6,"Exceeds Expectations",
  IF(E16&gt;=2,"Meets Expectations","Needs Improvement")))</f>
-        <v>Exceeds Expectations</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A17" s="9" t="str">
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6">
+      <c r="A17" s="9">
         <f>A4</f>
-        <v>patricia</v>
+        <v>0</v>
       </c>
       <c r="B17" s="10">
         <f t="shared" si="1"/>
-        <v>2.0499999999999998</v>
+        <v>0</v>
       </c>
       <c r="C17" s="10">
         <f t="shared" si="1"/>
-        <v>2.13</v>
-      </c>
-      <c r="D17" s="10">
+        <v>0</v>
+      </c>
+      <c r="D17" s="10" t="e">
         <f t="shared" ref="D17:D18" si="2">$C$11</f>
-        <v>2.38</v>
-      </c>
-      <c r="E17" s="14">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="E17" s="14" t="e">
         <f>B17*$E$1+D17*$G$1</f>
-        <v>2.1159999999999997</v>
-      </c>
-      <c r="F17" s="9" t="str">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="F17" s="9" t="e">
         <f t="shared" ref="F17:F18" si="3">IF(E17&gt;=3.6,"Outstanding",
  IF(E17&gt;=2.6,"Exceeds Expectations",
  IF(E17&gt;=2,"Meets Expectations","Needs Improvement")))</f>
-        <v>Meets Expectations</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A18" s="9" t="str">
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6">
+      <c r="A18" s="9">
         <f>A5</f>
-        <v>miguel</v>
+        <v>0</v>
       </c>
       <c r="B18" s="10">
         <f t="shared" si="1"/>
@@ -990,20 +957,20 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="D18" s="10">
+      <c r="D18" s="10" t="e">
         <f t="shared" si="2"/>
-        <v>2.38</v>
-      </c>
-      <c r="E18" s="14">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="E18" s="14" t="e">
         <f>B18*$E$1+D18*$G$1</f>
-        <v>0.47599999999999998</v>
-      </c>
-      <c r="F18" s="9" t="str">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="F18" s="9" t="e">
         <f t="shared" si="3"/>
-        <v>Needs Improvement</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6">
       <c r="A19" s="9"/>
       <c r="B19" s="10"/>
       <c r="C19" s="10"/>
@@ -1011,7 +978,7 @@
       <c r="E19" s="14"/>
       <c r="F19" s="9"/>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6">
       <c r="A20" s="9"/>
       <c r="B20" s="10"/>
       <c r="C20" s="10"/>

</xml_diff>

<commit_message>
Enhance user management and evaluation processes by adding eligibility checks for HRIS accounts, refining data retrieval for employee roles, and implementing filtering options in evaluation history. Update SQL scripts for President/CEO accounts and probationary templates.
</commit_message>
<xml_diff>
--- a/Raquel_Pawnshop_HR_Workforce_Analytics_&_Evaluation _Platform-Computation.xlsx
+++ b/Raquel_Pawnshop_HR_Workforce_Analytics_&_Evaluation _Platform-Computation.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\Raquel_HRD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{642FECBF-AB68-40BB-A10A-A0182D274CE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0F1F6BD-C03F-432F-9915-C64CD5D400EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{22A5745B-9E59-4E91-9FA4-3C7DB1ABBFEE}"/>
   </bookViews>
@@ -142,7 +142,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -701,18 +701,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A83BB1C1-F953-4E33-A206-594A5C40587D}">
   <dimension ref="A1:H20"/>
-  <sheetFormatPr defaultColWidth="26" defaultRowHeight="14"/>
+  <sheetFormatPr defaultColWidth="26" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="52.1640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.75" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="20.4140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.58203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.83203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.58203125" customWidth="1"/>
+    <col min="1" max="1" width="52.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.7265625" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="20.453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.54296875" customWidth="1"/>
     <col min="8" max="8" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
@@ -733,7 +733,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="14.5">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" s="11" t="s">
         <v>4</v>
       </c>
@@ -755,27 +755,31 @@
       <c r="G2" s="1"/>
       <c r="H2" s="1"/>
     </row>
-    <row r="3" spans="1:8" ht="16">
+    <row r="3" spans="1:8" ht="16" x14ac:dyDescent="0.45">
       <c r="A3" s="18" t="s">
         <v>18</v>
       </c>
       <c r="B3" s="16"/>
-      <c r="C3" s="17"/>
-      <c r="D3" s="17"/>
+      <c r="C3" s="17">
+        <v>3.35</v>
+      </c>
+      <c r="D3" s="17">
+        <v>3.5</v>
+      </c>
       <c r="E3" s="7">
         <f>C3*$E$1+D3*$G$1</f>
-        <v>0</v>
+        <v>3.3800000000000003</v>
       </c>
       <c r="F3" s="6" t="str">
         <f>IF(E3&gt;=3.6,"Outstanding",
  IF(E3&gt;=2.6,"Exceeds Expectations",
  IF(E3&gt;=2,"Meets Expectations","Needs Improvement")))</f>
-        <v>Needs Improvement</v>
+        <v>Exceeds Expectations</v>
       </c>
       <c r="G3" s="1"/>
       <c r="H3" s="1"/>
     </row>
-    <row r="4" spans="1:8" ht="16">
+    <row r="4" spans="1:8" ht="16" x14ac:dyDescent="0.45">
       <c r="A4" s="18"/>
       <c r="B4" s="16"/>
       <c r="C4" s="17"/>
@@ -793,7 +797,7 @@
       <c r="G4" s="1"/>
       <c r="H4" s="1"/>
     </row>
-    <row r="5" spans="1:8" ht="16">
+    <row r="5" spans="1:8" ht="16" x14ac:dyDescent="0.45">
       <c r="A5" s="18"/>
       <c r="B5" s="16"/>
       <c r="C5" s="17"/>
@@ -809,7 +813,7 @@
       <c r="G5" s="1"/>
       <c r="H5" s="1"/>
     </row>
-    <row r="6" spans="1:8" ht="16">
+    <row r="6" spans="1:8" ht="16" x14ac:dyDescent="0.45">
       <c r="A6" s="18"/>
       <c r="B6" s="16"/>
       <c r="C6" s="17"/>
@@ -817,7 +821,7 @@
       <c r="E6" s="6"/>
       <c r="F6" s="19"/>
     </row>
-    <row r="7" spans="1:8" ht="16">
+    <row r="7" spans="1:8" ht="16" x14ac:dyDescent="0.45">
       <c r="A7" s="18"/>
       <c r="B7" s="16"/>
       <c r="C7" s="17"/>
@@ -825,12 +829,12 @@
       <c r="E7" s="6"/>
       <c r="F7" s="19"/>
     </row>
-    <row r="8" spans="1:8">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="14.5">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A10" s="8" t="s">
         <v>7</v>
       </c>
@@ -841,7 +845,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:8">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="s">
         <v>10</v>
       </c>
@@ -849,24 +853,24 @@
         <f>COUNTA(A3:A7)</f>
         <v>1</v>
       </c>
-      <c r="C11" s="10" t="e">
+      <c r="C11" s="10">
         <f>AVERAGE(D3:D7)</f>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A12" s="1"/>
       <c r="B12" s="1"/>
       <c r="C12" s="1"/>
     </row>
-    <row r="13" spans="1:8" ht="14.5">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
         <v>11</v>
       </c>
       <c r="B13" s="4"/>
       <c r="C13" s="5"/>
     </row>
-    <row r="15" spans="1:8" ht="14.5">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A15" s="13" t="s">
         <v>4</v>
       </c>
@@ -888,35 +892,35 @@
         <v>13</v>
       </c>
     </row>
-    <row r="16" spans="1:8">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A16" s="9" t="str">
         <f>A3</f>
         <v>liana</v>
       </c>
       <c r="B16" s="10">
         <f t="shared" ref="B16:C18" si="1">C3</f>
-        <v>0</v>
+        <v>3.35</v>
       </c>
       <c r="C16" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="D16" s="10" t="e">
+        <v>3.5</v>
+      </c>
+      <c r="D16" s="10">
         <f>$C$11</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E16" s="14" t="e">
+        <v>3.5</v>
+      </c>
+      <c r="E16" s="14">
         <f>B16*$E$1+D16*$G$1</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F16" s="9" t="e">
+        <v>3.3800000000000003</v>
+      </c>
+      <c r="F16" s="9" t="str">
         <f>IF(E16&gt;=3.6,"Outstanding",
  IF(E16&gt;=2.6,"Exceeds Expectations",
  IF(E16&gt;=2,"Meets Expectations","Needs Improvement")))</f>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6">
+        <v>Exceeds Expectations</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17" s="9">
         <f>A4</f>
         <v>0</v>
@@ -929,22 +933,22 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="D17" s="10" t="e">
+      <c r="D17" s="10">
         <f t="shared" ref="D17:D18" si="2">$C$11</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E17" s="14" t="e">
+        <v>3.5</v>
+      </c>
+      <c r="E17" s="14">
         <f>B17*$E$1+D17*$G$1</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F17" s="9" t="e">
+        <v>0.70000000000000007</v>
+      </c>
+      <c r="F17" s="9" t="str">
         <f t="shared" ref="F17:F18" si="3">IF(E17&gt;=3.6,"Outstanding",
  IF(E17&gt;=2.6,"Exceeds Expectations",
  IF(E17&gt;=2,"Meets Expectations","Needs Improvement")))</f>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6">
+        <v>Needs Improvement</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A18" s="9">
         <f>A5</f>
         <v>0</v>
@@ -957,20 +961,20 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="D18" s="10" t="e">
+      <c r="D18" s="10">
         <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E18" s="14" t="e">
+        <v>3.5</v>
+      </c>
+      <c r="E18" s="14">
         <f>B18*$E$1+D18*$G$1</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F18" s="9" t="e">
+        <v>0.70000000000000007</v>
+      </c>
+      <c r="F18" s="9" t="str">
         <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6">
+        <v>Needs Improvement</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19" s="9"/>
       <c r="B19" s="10"/>
       <c r="C19" s="10"/>
@@ -978,7 +982,7 @@
       <c r="E19" s="14"/>
       <c r="F19" s="9"/>
     </row>
-    <row r="20" spans="1:6">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20" s="9"/>
       <c r="B20" s="10"/>
       <c r="C20" s="10"/>

</xml_diff>

<commit_message>
Update HR Workforce Analytics and Evaluation computation file
</commit_message>
<xml_diff>
--- a/Raquel_Pawnshop_HR_Workforce_Analytics_&_Evaluation _Platform-Computation.xlsx
+++ b/Raquel_Pawnshop_HR_Workforce_Analytics_&_Evaluation _Platform-Computation.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\Raquel_HRD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0F1F6BD-C03F-432F-9915-C64CD5D400EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CC406AD-92B6-4BCA-88E4-AF99AAA4871B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{22A5745B-9E59-4E91-9FA4-3C7DB1ABBFEE}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="auto" sheetId="1" r:id="rId1"/>
+    <sheet name="manual" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -52,7 +53,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">Average of Self Core Values within the department
 </t>
@@ -67,7 +68,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">Final Score absorbed by the system
 </t>
@@ -79,7 +80,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="50">
   <si>
     <t>Rating Scale</t>
   </si>
@@ -136,13 +137,106 @@
   </si>
   <si>
     <t>liana</t>
+  </si>
+  <si>
+    <t>KRA Items</t>
+  </si>
+  <si>
+    <t>Weight</t>
+  </si>
+  <si>
+    <t>Core Behavior &amp; values</t>
+  </si>
+  <si>
+    <t>KRA 1</t>
+  </si>
+  <si>
+    <t>Core Item 1</t>
+  </si>
+  <si>
+    <t>KRA 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Core Item 2 </t>
+  </si>
+  <si>
+    <t>KRA 3</t>
+  </si>
+  <si>
+    <t>Core Item 3</t>
+  </si>
+  <si>
+    <t>KRA 4</t>
+  </si>
+  <si>
+    <t>Core Item 4</t>
+  </si>
+  <si>
+    <t>KRA 5</t>
+  </si>
+  <si>
+    <t>Core Item 5</t>
+  </si>
+  <si>
+    <t>KRA 6</t>
+  </si>
+  <si>
+    <t>Core Item 6</t>
+  </si>
+  <si>
+    <t>KRA 7</t>
+  </si>
+  <si>
+    <t>Core Item 7</t>
+  </si>
+  <si>
+    <t>KRA 8</t>
+  </si>
+  <si>
+    <t>Core Item 8</t>
+  </si>
+  <si>
+    <t>KRA 9</t>
+  </si>
+  <si>
+    <t>KRA 10</t>
+  </si>
+  <si>
+    <t>KRA 11</t>
+  </si>
+  <si>
+    <t>KRA 12</t>
+  </si>
+  <si>
+    <t>KRA 13</t>
+  </si>
+  <si>
+    <t>KRA 14</t>
+  </si>
+  <si>
+    <t>KRA 15</t>
+  </si>
+  <si>
+    <t>KRA 16</t>
+  </si>
+  <si>
+    <t>KRA 17</t>
+  </si>
+  <si>
+    <t>KRA Subtotal</t>
+  </si>
+  <si>
+    <t>Core Values Average</t>
+  </si>
+  <si>
+    <t>Core Values Weight</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -162,6 +256,7 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -194,7 +289,12 @@
       <sz val="9"/>
       <color indexed="81"/>
       <name val="Tahoma"/>
-      <charset val="1"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
     </font>
   </fonts>
   <fills count="7">
@@ -309,7 +409,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -366,6 +466,15 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="9" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -701,7 +810,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A83BB1C1-F953-4E33-A206-594A5C40587D}">
   <dimension ref="A1:H20"/>
-  <sheetFormatPr defaultColWidth="26" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="26" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="52.1796875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10.7265625" bestFit="1" customWidth="1"/>
@@ -712,7 +821,7 @@
     <col min="8" max="8" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8">
       <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
@@ -733,7 +842,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8">
       <c r="A2" s="11" t="s">
         <v>4</v>
       </c>
@@ -755,20 +864,20 @@
       <c r="G2" s="1"/>
       <c r="H2" s="1"/>
     </row>
-    <row r="3" spans="1:8" ht="16" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:8" ht="16">
       <c r="A3" s="18" t="s">
         <v>18</v>
       </c>
       <c r="B3" s="16"/>
-      <c r="C3" s="17">
-        <v>3.35</v>
+      <c r="C3">
+        <v>3.36</v>
       </c>
       <c r="D3" s="17">
-        <v>3.5</v>
+        <v>3.13</v>
       </c>
       <c r="E3" s="7">
         <f>C3*$E$1+D3*$G$1</f>
-        <v>3.3800000000000003</v>
+        <v>3.3140000000000001</v>
       </c>
       <c r="F3" s="6" t="str">
         <f>IF(E3&gt;=3.6,"Outstanding",
@@ -779,7 +888,7 @@
       <c r="G3" s="1"/>
       <c r="H3" s="1"/>
     </row>
-    <row r="4" spans="1:8" ht="16" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:8" ht="16">
       <c r="A4" s="18"/>
       <c r="B4" s="16"/>
       <c r="C4" s="17"/>
@@ -797,7 +906,7 @@
       <c r="G4" s="1"/>
       <c r="H4" s="1"/>
     </row>
-    <row r="5" spans="1:8" ht="16" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:8" ht="16">
       <c r="A5" s="18"/>
       <c r="B5" s="16"/>
       <c r="C5" s="17"/>
@@ -813,7 +922,7 @@
       <c r="G5" s="1"/>
       <c r="H5" s="1"/>
     </row>
-    <row r="6" spans="1:8" ht="16" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:8" ht="16">
       <c r="A6" s="18"/>
       <c r="B6" s="16"/>
       <c r="C6" s="17"/>
@@ -821,7 +930,7 @@
       <c r="E6" s="6"/>
       <c r="F6" s="19"/>
     </row>
-    <row r="7" spans="1:8" ht="16" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:8" ht="16">
       <c r="A7" s="18"/>
       <c r="B7" s="16"/>
       <c r="C7" s="17"/>
@@ -829,12 +938,12 @@
       <c r="E7" s="6"/>
       <c r="F7" s="19"/>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:8">
       <c r="A8" s="2" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:8">
       <c r="A10" s="8" t="s">
         <v>7</v>
       </c>
@@ -845,7 +954,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:8">
       <c r="A11" s="9" t="s">
         <v>10</v>
       </c>
@@ -855,22 +964,22 @@
       </c>
       <c r="C11" s="10">
         <f>AVERAGE(D3:D7)</f>
-        <v>3.5</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+        <v>3.13</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8">
       <c r="A12" s="1"/>
       <c r="B12" s="1"/>
       <c r="C12" s="1"/>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:8">
       <c r="A13" s="3" t="s">
         <v>11</v>
       </c>
       <c r="B13" s="4"/>
       <c r="C13" s="5"/>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:8">
       <c r="A15" s="13" t="s">
         <v>4</v>
       </c>
@@ -892,26 +1001,26 @@
         <v>13</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:8">
       <c r="A16" s="9" t="str">
         <f>A3</f>
         <v>liana</v>
       </c>
       <c r="B16" s="10">
         <f t="shared" ref="B16:C18" si="1">C3</f>
-        <v>3.35</v>
+        <v>3.36</v>
       </c>
       <c r="C16" s="10">
         <f t="shared" si="1"/>
-        <v>3.5</v>
+        <v>3.13</v>
       </c>
       <c r="D16" s="10">
         <f>$C$11</f>
-        <v>3.5</v>
+        <v>3.13</v>
       </c>
       <c r="E16" s="14">
         <f>B16*$E$1+D16*$G$1</f>
-        <v>3.3800000000000003</v>
+        <v>3.3140000000000001</v>
       </c>
       <c r="F16" s="9" t="str">
         <f>IF(E16&gt;=3.6,"Outstanding",
@@ -920,7 +1029,7 @@
         <v>Exceeds Expectations</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:6">
       <c r="A17" s="9">
         <f>A4</f>
         <v>0</v>
@@ -935,11 +1044,11 @@
       </c>
       <c r="D17" s="10">
         <f t="shared" ref="D17:D18" si="2">$C$11</f>
-        <v>3.5</v>
+        <v>3.13</v>
       </c>
       <c r="E17" s="14">
         <f>B17*$E$1+D17*$G$1</f>
-        <v>0.70000000000000007</v>
+        <v>0.626</v>
       </c>
       <c r="F17" s="9" t="str">
         <f t="shared" ref="F17:F18" si="3">IF(E17&gt;=3.6,"Outstanding",
@@ -948,7 +1057,7 @@
         <v>Needs Improvement</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:6">
       <c r="A18" s="9">
         <f>A5</f>
         <v>0</v>
@@ -963,18 +1072,18 @@
       </c>
       <c r="D18" s="10">
         <f t="shared" si="2"/>
-        <v>3.5</v>
+        <v>3.13</v>
       </c>
       <c r="E18" s="14">
         <f>B18*$E$1+D18*$G$1</f>
-        <v>0.70000000000000007</v>
+        <v>0.626</v>
       </c>
       <c r="F18" s="9" t="str">
         <f t="shared" si="3"/>
         <v>Needs Improvement</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:6">
       <c r="A19" s="9"/>
       <c r="B19" s="10"/>
       <c r="C19" s="10"/>
@@ -982,7 +1091,7 @@
       <c r="E19" s="14"/>
       <c r="F19" s="9"/>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:6">
       <c r="A20" s="9"/>
       <c r="B20" s="10"/>
       <c r="C20" s="10"/>
@@ -995,4 +1104,326 @@
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <legacyDrawing r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BA4D037B-B578-4EA5-923C-168A9DE23B26}">
+  <dimension ref="A1:L19"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
+  <cols>
+    <col min="1" max="1" width="8.90625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="5.90625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.36328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="5.90625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.08984375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="16.6328125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="9.7265625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12">
+      <c r="A1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H1" t="s">
+        <v>47</v>
+      </c>
+      <c r="I1" t="s">
+        <v>48</v>
+      </c>
+      <c r="J1" t="s">
+        <v>2</v>
+      </c>
+      <c r="K1" t="s">
+        <v>49</v>
+      </c>
+      <c r="L1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12">
+      <c r="A2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B2" s="20">
+        <v>0.05</v>
+      </c>
+      <c r="C2">
+        <v>2</v>
+      </c>
+      <c r="E2" t="s">
+        <v>23</v>
+      </c>
+      <c r="F2">
+        <v>4</v>
+      </c>
+      <c r="H2" s="24">
+        <f>SUMPRODUCT(B2:B18,C2:C18)</f>
+        <v>3.3600000000000008</v>
+      </c>
+      <c r="I2" s="21">
+        <f>F10/8</f>
+        <v>3.125</v>
+      </c>
+      <c r="J2" s="22">
+        <v>0.8</v>
+      </c>
+      <c r="K2" s="22">
+        <v>0.2</v>
+      </c>
+      <c r="L2" s="21">
+        <f>(H2*J2)+(I2*K2)</f>
+        <v>3.3130000000000006</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12">
+      <c r="A3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B3" s="20">
+        <v>0.1</v>
+      </c>
+      <c r="C3">
+        <v>3</v>
+      </c>
+      <c r="E3" t="s">
+        <v>25</v>
+      </c>
+      <c r="F3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12">
+      <c r="A4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B4" s="20">
+        <v>0.05</v>
+      </c>
+      <c r="C4">
+        <v>4</v>
+      </c>
+      <c r="E4" t="s">
+        <v>27</v>
+      </c>
+      <c r="F4">
+        <v>3</v>
+      </c>
+      <c r="I4" s="21"/>
+    </row>
+    <row r="5" spans="1:12">
+      <c r="A5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B5" s="20">
+        <v>0.05</v>
+      </c>
+      <c r="C5">
+        <v>3</v>
+      </c>
+      <c r="E5" t="s">
+        <v>29</v>
+      </c>
+      <c r="F5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12">
+      <c r="A6" t="s">
+        <v>30</v>
+      </c>
+      <c r="B6" s="20">
+        <v>0.05</v>
+      </c>
+      <c r="C6">
+        <v>4</v>
+      </c>
+      <c r="E6" t="s">
+        <v>31</v>
+      </c>
+      <c r="F6">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12">
+      <c r="A7" t="s">
+        <v>32</v>
+      </c>
+      <c r="B7" s="20">
+        <v>0.2</v>
+      </c>
+      <c r="C7">
+        <v>4</v>
+      </c>
+      <c r="E7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F7">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12">
+      <c r="A8" t="s">
+        <v>34</v>
+      </c>
+      <c r="B8" s="20">
+        <v>0.1</v>
+      </c>
+      <c r="C8">
+        <v>4</v>
+      </c>
+      <c r="E8" t="s">
+        <v>35</v>
+      </c>
+      <c r="F8">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12">
+      <c r="A9" t="s">
+        <v>36</v>
+      </c>
+      <c r="B9" s="20">
+        <v>0.02</v>
+      </c>
+      <c r="C9">
+        <v>4</v>
+      </c>
+      <c r="E9" t="s">
+        <v>37</v>
+      </c>
+      <c r="F9">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12">
+      <c r="A10" t="s">
+        <v>38</v>
+      </c>
+      <c r="B10" s="20">
+        <v>0.03</v>
+      </c>
+      <c r="C10">
+        <v>3</v>
+      </c>
+      <c r="F10" s="23">
+        <f>SUM(F2:F9)</f>
+        <v>25</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12">
+      <c r="A11" t="s">
+        <v>39</v>
+      </c>
+      <c r="B11" s="20">
+        <v>0.05</v>
+      </c>
+      <c r="C11">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12">
+      <c r="A12" t="s">
+        <v>40</v>
+      </c>
+      <c r="B12" s="20">
+        <v>0.03</v>
+      </c>
+      <c r="C12">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12">
+      <c r="A13" t="s">
+        <v>41</v>
+      </c>
+      <c r="B13" s="20">
+        <v>0.02</v>
+      </c>
+      <c r="C13">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12">
+      <c r="A14" t="s">
+        <v>42</v>
+      </c>
+      <c r="B14" s="20">
+        <v>0.05</v>
+      </c>
+      <c r="C14">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12">
+      <c r="A15" t="s">
+        <v>43</v>
+      </c>
+      <c r="B15" s="20">
+        <v>0.05</v>
+      </c>
+      <c r="C15">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12">
+      <c r="A16" t="s">
+        <v>44</v>
+      </c>
+      <c r="B16" s="20">
+        <v>0.05</v>
+      </c>
+      <c r="C16">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3">
+      <c r="A17" t="s">
+        <v>45</v>
+      </c>
+      <c r="B17" s="20">
+        <v>0.05</v>
+      </c>
+      <c r="C17">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3">
+      <c r="A18" t="s">
+        <v>46</v>
+      </c>
+      <c r="B18" s="20">
+        <v>0.05</v>
+      </c>
+      <c r="C18">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3">
+      <c r="B19" s="22">
+        <f>SUM(B2:B18)</f>
+        <v>1.0000000000000002</v>
+      </c>
+      <c r="C19" s="23">
+        <f>SUM(C2:C18)</f>
+        <v>55</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add annual evaluation functionality and related templates
- Introduced annual-template-controls.php for core values and JS integration.
- Created performance-evaluation-heading.php for shared HRIS headings and evaluation categories.
- Added annual-evaluations.php for HR Manager, Staff, and Supervisor roles with session checks and role validation.
- Implemented tests for annual evaluations, including database setup, evaluation creation, and validation of various scenarios.
- Developed annual-request.php for isolated controller requests to handle template creation and submission processes.
</commit_message>
<xml_diff>
--- a/Raquel_Pawnshop_HR_Workforce_Analytics_&_Evaluation _Platform-Computation.xlsx
+++ b/Raquel_Pawnshop_HR_Workforce_Analytics_&_Evaluation _Platform-Computation.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\Raquel_HRD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CC406AD-92B6-4BCA-88E4-AF99AAA4871B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83062282-663D-4988-9AEF-66FA45862314}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{22A5745B-9E59-4E91-9FA4-3C7DB1ABBFEE}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" activeTab="1" xr2:uid="{22A5745B-9E59-4E91-9FA4-3C7DB1ABBFEE}"/>
   </bookViews>
   <sheets>
     <sheet name="auto" sheetId="1" r:id="rId1"/>
     <sheet name="manual" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet1" sheetId="4" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -80,7 +81,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="72">
   <si>
     <t>Rating Scale</t>
   </si>
@@ -136,9 +137,6 @@
     <t>Score</t>
   </si>
   <si>
-    <t>liana</t>
-  </si>
-  <si>
     <t>KRA Items</t>
   </si>
   <si>
@@ -230,6 +228,75 @@
   </si>
   <si>
     <t>Core Values Weight</t>
+  </si>
+  <si>
+    <t>hr manager</t>
+  </si>
+  <si>
+    <t>hr supervisor</t>
+  </si>
+  <si>
+    <t>hr staff</t>
+  </si>
+  <si>
+    <t>Elena</t>
+  </si>
+  <si>
+    <t>Patricia</t>
+  </si>
+  <si>
+    <t>Miguel</t>
+  </si>
+  <si>
+    <t>kra score</t>
+  </si>
+  <si>
+    <t>self core behaviors</t>
+  </si>
+  <si>
+    <t>score</t>
+  </si>
+  <si>
+    <t>employee</t>
+  </si>
+  <si>
+    <t>HR Manager Rates</t>
+  </si>
+  <si>
+    <t>HR Supervisor Rates</t>
+  </si>
+  <si>
+    <t>HR Staff Rates</t>
+  </si>
+  <si>
+    <t>HR Manager</t>
+  </si>
+  <si>
+    <t>HR Supervisor</t>
+  </si>
+  <si>
+    <t>HR Staff</t>
+  </si>
+  <si>
+    <t>Employee Being Rated BAHAVIOR</t>
+  </si>
+  <si>
+    <t>AVERAGE</t>
+  </si>
+  <si>
+    <t>peer 360 rating</t>
+  </si>
+  <si>
+    <t>final result/score</t>
+  </si>
+  <si>
+    <t xml:space="preserve">THIS IS THE INITIAL PROCESS FOR SELF RATING </t>
+  </si>
+  <si>
+    <t>THIS IS THE BEHAVIOR 360 RATING (PEERS)</t>
+  </si>
+  <si>
+    <t>THIS IS THE SYSTEM MUST ABSORBED</t>
   </si>
 </sst>
 </file>
@@ -297,7 +364,7 @@
       <name val="Arial Unicode MS"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="12">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -328,6 +395,36 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.39997558519241921"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -409,7 +506,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -473,6 +570,54 @@
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="9" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="10" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="9" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="8" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="11" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -866,58 +1011,76 @@
     </row>
     <row r="3" spans="1:8" ht="16">
       <c r="A3" s="18" t="s">
-        <v>18</v>
-      </c>
-      <c r="B3" s="16"/>
-      <c r="C3">
-        <v>3.36</v>
+        <v>52</v>
+      </c>
+      <c r="B3" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="C3" s="25">
+        <v>3.9</v>
       </c>
       <c r="D3" s="17">
-        <v>3.13</v>
+        <v>3.6</v>
       </c>
       <c r="E3" s="7">
         <f>C3*$E$1+D3*$G$1</f>
-        <v>3.3140000000000001</v>
+        <v>3.8400000000000003</v>
       </c>
       <c r="F3" s="6" t="str">
         <f>IF(E3&gt;=3.6,"Outstanding",
  IF(E3&gt;=2.6,"Exceeds Expectations",
  IF(E3&gt;=2,"Meets Expectations","Needs Improvement")))</f>
-        <v>Exceeds Expectations</v>
+        <v>Outstanding</v>
       </c>
       <c r="G3" s="1"/>
       <c r="H3" s="1"/>
     </row>
     <row r="4" spans="1:8" ht="16">
-      <c r="A4" s="18"/>
-      <c r="B4" s="16"/>
-      <c r="C4" s="17"/>
-      <c r="D4" s="17"/>
+      <c r="A4" s="18" t="s">
+        <v>53</v>
+      </c>
+      <c r="B4" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="C4" s="17">
+        <v>3.2</v>
+      </c>
+      <c r="D4" s="17">
+        <v>3.4</v>
+      </c>
       <c r="E4" s="7">
         <f>C4*$E$1+D4*$G$1</f>
-        <v>0</v>
+        <v>3.2400000000000007</v>
       </c>
       <c r="F4" s="6" t="str">
         <f t="shared" ref="F4:F5" si="0">IF(E4&gt;=3.6,"Outstanding",
  IF(E4&gt;=2.6,"Exceeds Expectations",
  IF(E4&gt;=2,"Meets Expectations","Needs Improvement")))</f>
-        <v>Needs Improvement</v>
+        <v>Exceeds Expectations</v>
       </c>
       <c r="G4" s="1"/>
       <c r="H4" s="1"/>
     </row>
     <row r="5" spans="1:8" ht="16">
-      <c r="A5" s="18"/>
-      <c r="B5" s="16"/>
-      <c r="C5" s="17"/>
-      <c r="D5" s="17"/>
+      <c r="A5" s="18" t="s">
+        <v>54</v>
+      </c>
+      <c r="B5" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="C5" s="17">
+        <v>2.4</v>
+      </c>
+      <c r="D5" s="17">
+        <v>4</v>
+      </c>
       <c r="E5" s="7">
         <f>C5*$E$1+D5*$G$1</f>
-        <v>0</v>
+        <v>2.7199999999999998</v>
       </c>
       <c r="F5" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>Needs Improvement</v>
+        <v>Exceeds Expectations</v>
       </c>
       <c r="G5" s="1"/>
       <c r="H5" s="1"/>
@@ -960,11 +1123,11 @@
       </c>
       <c r="B11" s="9">
         <f>COUNTA(A3:A7)</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C11" s="10">
         <f>AVERAGE(D3:D7)</f>
-        <v>3.13</v>
+        <v>3.6666666666666665</v>
       </c>
     </row>
     <row r="12" spans="1:8">
@@ -1004,83 +1167,83 @@
     <row r="16" spans="1:8">
       <c r="A16" s="9" t="str">
         <f>A3</f>
-        <v>liana</v>
+        <v>Elena</v>
       </c>
       <c r="B16" s="10">
         <f t="shared" ref="B16:C18" si="1">C3</f>
-        <v>3.36</v>
+        <v>3.9</v>
       </c>
       <c r="C16" s="10">
         <f t="shared" si="1"/>
-        <v>3.13</v>
+        <v>3.6</v>
       </c>
       <c r="D16" s="10">
         <f>$C$11</f>
-        <v>3.13</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="E16" s="14">
         <f>B16*$E$1+D16*$G$1</f>
-        <v>3.3140000000000001</v>
+        <v>3.8533333333333335</v>
       </c>
       <c r="F16" s="9" t="str">
         <f>IF(E16&gt;=3.6,"Outstanding",
  IF(E16&gt;=2.6,"Exceeds Expectations",
  IF(E16&gt;=2,"Meets Expectations","Needs Improvement")))</f>
-        <v>Exceeds Expectations</v>
+        <v>Outstanding</v>
       </c>
     </row>
     <row r="17" spans="1:6">
-      <c r="A17" s="9">
+      <c r="A17" s="9" t="str">
         <f>A4</f>
-        <v>0</v>
+        <v>Patricia</v>
       </c>
       <c r="B17" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>3.2</v>
       </c>
       <c r="C17" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>3.4</v>
       </c>
       <c r="D17" s="10">
         <f t="shared" ref="D17:D18" si="2">$C$11</f>
-        <v>3.13</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="E17" s="14">
         <f>B17*$E$1+D17*$G$1</f>
-        <v>0.626</v>
+        <v>3.2933333333333339</v>
       </c>
       <c r="F17" s="9" t="str">
         <f t="shared" ref="F17:F18" si="3">IF(E17&gt;=3.6,"Outstanding",
  IF(E17&gt;=2.6,"Exceeds Expectations",
  IF(E17&gt;=2,"Meets Expectations","Needs Improvement")))</f>
-        <v>Needs Improvement</v>
+        <v>Exceeds Expectations</v>
       </c>
     </row>
     <row r="18" spans="1:6">
-      <c r="A18" s="9">
+      <c r="A18" s="9" t="str">
         <f>A5</f>
-        <v>0</v>
+        <v>Miguel</v>
       </c>
       <c r="B18" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>2.4</v>
       </c>
       <c r="C18" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D18" s="10">
         <f t="shared" si="2"/>
-        <v>3.13</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="E18" s="14">
         <f>B18*$E$1+D18*$G$1</f>
-        <v>0.626</v>
+        <v>2.6533333333333333</v>
       </c>
       <c r="F18" s="9" t="str">
         <f t="shared" si="3"/>
-        <v>Needs Improvement</v>
+        <v>Exceeds Expectations</v>
       </c>
     </row>
     <row r="19" spans="1:6">
@@ -1108,12 +1271,9 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BA4D037B-B578-4EA5-923C-168A9DE23B26}">
-  <dimension ref="A1:L19"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <dimension ref="A1:N19"/>
+  <sheetFormatPr defaultColWidth="7" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="8.90625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.453125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="5.90625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="19.36328125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="5.90625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="11.08984375" bestFit="1" customWidth="1"/>
@@ -1123,57 +1283,58 @@
     <col min="12" max="12" width="9.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12">
+    <row r="1" spans="1:14">
       <c r="A1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B1" t="s">
         <v>19</v>
-      </c>
-      <c r="B1" t="s">
-        <v>20</v>
       </c>
       <c r="C1" t="s">
         <v>13</v>
       </c>
       <c r="E1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F1" t="s">
         <v>13</v>
       </c>
       <c r="H1" t="s">
+        <v>46</v>
+      </c>
+      <c r="I1" t="s">
         <v>47</v>
-      </c>
-      <c r="I1" t="s">
-        <v>48</v>
       </c>
       <c r="J1" t="s">
         <v>2</v>
       </c>
       <c r="K1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="L1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:12">
+    <row r="2" spans="1:14">
       <c r="A2" t="s">
-        <v>22</v>
-      </c>
-      <c r="B2" s="20">
+        <v>21</v>
+      </c>
+      <c r="B2" s="42">
         <v>0.05</v>
       </c>
       <c r="C2">
         <v>2</v>
       </c>
+      <c r="D2" s="40"/>
       <c r="E2" t="s">
-        <v>23</v>
-      </c>
-      <c r="F2">
+        <v>22</v>
+      </c>
+      <c r="F2" s="24">
         <v>4</v>
       </c>
-      <c r="H2" s="24">
+      <c r="H2" s="41">
         <f>SUMPRODUCT(B2:B18,C2:C18)</f>
-        <v>3.3600000000000008</v>
+        <v>3.3900000000000006</v>
       </c>
       <c r="I2" s="21">
         <f>F10/8</f>
@@ -1187,233 +1348,283 @@
       </c>
       <c r="L2" s="21">
         <f>(H2*J2)+(I2*K2)</f>
-        <v>3.3130000000000006</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12">
+        <v>3.3370000000000006</v>
+      </c>
+      <c r="M2" s="20"/>
+      <c r="N2" s="42"/>
+    </row>
+    <row r="3" spans="1:14">
       <c r="A3" t="s">
-        <v>24</v>
-      </c>
-      <c r="B3" s="20">
+        <v>23</v>
+      </c>
+      <c r="B3" s="42">
         <v>0.1</v>
       </c>
       <c r="C3">
         <v>3</v>
       </c>
+      <c r="D3" s="40"/>
       <c r="E3" t="s">
+        <v>24</v>
+      </c>
+      <c r="F3" s="24">
+        <v>4</v>
+      </c>
+      <c r="M3" s="20"/>
+      <c r="N3" s="42"/>
+    </row>
+    <row r="4" spans="1:14">
+      <c r="A4" t="s">
         <v>25</v>
       </c>
-      <c r="F3">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12">
-      <c r="A4" t="s">
-        <v>26</v>
-      </c>
-      <c r="B4" s="20">
+      <c r="B4" s="42">
         <v>0.05</v>
       </c>
       <c r="C4">
         <v>4</v>
       </c>
+      <c r="D4" s="40"/>
       <c r="E4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F4" s="24">
+        <v>3</v>
+      </c>
+      <c r="I4" s="21"/>
+      <c r="M4" s="20"/>
+      <c r="N4" s="42"/>
+    </row>
+    <row r="5" spans="1:14">
+      <c r="A5" t="s">
         <v>27</v>
       </c>
-      <c r="F4">
-        <v>3</v>
-      </c>
-      <c r="I4" s="21"/>
-    </row>
-    <row r="5" spans="1:12">
-      <c r="A5" t="s">
-        <v>28</v>
-      </c>
-      <c r="B5" s="20">
+      <c r="B5" s="42">
         <v>0.05</v>
       </c>
       <c r="C5">
         <v>3</v>
       </c>
+      <c r="D5" s="40"/>
       <c r="E5" t="s">
+        <v>28</v>
+      </c>
+      <c r="F5" s="24">
+        <v>2</v>
+      </c>
+      <c r="M5" s="20"/>
+      <c r="N5" s="42"/>
+    </row>
+    <row r="6" spans="1:14">
+      <c r="A6" t="s">
         <v>29</v>
       </c>
-      <c r="F5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12">
-      <c r="A6" t="s">
-        <v>30</v>
-      </c>
-      <c r="B6" s="20">
+      <c r="B6" s="42">
         <v>0.05</v>
       </c>
       <c r="C6">
         <v>4</v>
       </c>
+      <c r="D6" s="40"/>
       <c r="E6" t="s">
+        <v>30</v>
+      </c>
+      <c r="F6" s="24">
+        <v>2</v>
+      </c>
+      <c r="M6" s="20"/>
+      <c r="N6" s="42"/>
+    </row>
+    <row r="7" spans="1:14">
+      <c r="A7" t="s">
         <v>31</v>
       </c>
-      <c r="F6">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12">
-      <c r="A7" t="s">
-        <v>32</v>
-      </c>
-      <c r="B7" s="20">
-        <v>0.2</v>
+      <c r="B7" s="42">
+        <v>0.05</v>
       </c>
       <c r="C7">
         <v>4</v>
       </c>
+      <c r="D7" s="40"/>
       <c r="E7" t="s">
+        <v>32</v>
+      </c>
+      <c r="F7" s="24">
+        <v>3</v>
+      </c>
+      <c r="M7" s="20"/>
+      <c r="N7" s="42"/>
+    </row>
+    <row r="8" spans="1:14">
+      <c r="A8" t="s">
         <v>33</v>
       </c>
-      <c r="F7">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12">
-      <c r="A8" t="s">
-        <v>34</v>
-      </c>
-      <c r="B8" s="20">
-        <v>0.1</v>
+      <c r="B8" s="42">
+        <v>0.2</v>
       </c>
       <c r="C8">
         <v>4</v>
       </c>
+      <c r="D8" s="40"/>
       <c r="E8" t="s">
+        <v>34</v>
+      </c>
+      <c r="F8" s="24">
+        <v>3</v>
+      </c>
+      <c r="M8" s="20"/>
+      <c r="N8" s="42"/>
+    </row>
+    <row r="9" spans="1:14">
+      <c r="A9" t="s">
         <v>35</v>
       </c>
-      <c r="F8">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12">
-      <c r="A9" t="s">
-        <v>36</v>
-      </c>
-      <c r="B9" s="20">
-        <v>0.02</v>
+      <c r="B9" s="42">
+        <v>0.1</v>
       </c>
       <c r="C9">
         <v>4</v>
       </c>
+      <c r="D9" s="40"/>
       <c r="E9" t="s">
+        <v>36</v>
+      </c>
+      <c r="F9" s="24">
+        <v>4</v>
+      </c>
+      <c r="M9" s="20"/>
+      <c r="N9" s="42"/>
+    </row>
+    <row r="10" spans="1:14">
+      <c r="A10" t="s">
         <v>37</v>
       </c>
-      <c r="F9">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12">
-      <c r="A10" t="s">
-        <v>38</v>
-      </c>
-      <c r="B10" s="20">
-        <v>0.03</v>
+      <c r="B10" s="42">
+        <v>0.02</v>
       </c>
       <c r="C10">
         <v>3</v>
       </c>
+      <c r="D10" s="40"/>
       <c r="F10" s="23">
         <f>SUM(F2:F9)</f>
         <v>25</v>
       </c>
-    </row>
-    <row r="11" spans="1:12">
+      <c r="M10" s="20"/>
+      <c r="N10" s="42"/>
+    </row>
+    <row r="11" spans="1:14">
       <c r="A11" t="s">
-        <v>39</v>
-      </c>
-      <c r="B11" s="20">
-        <v>0.05</v>
+        <v>38</v>
+      </c>
+      <c r="B11" s="42">
+        <v>0.03</v>
       </c>
       <c r="C11">
         <v>3</v>
       </c>
-    </row>
-    <row r="12" spans="1:12">
+      <c r="D11" s="40"/>
+      <c r="M11" s="20"/>
+      <c r="N11" s="42"/>
+    </row>
+    <row r="12" spans="1:14">
       <c r="A12" t="s">
+        <v>39</v>
+      </c>
+      <c r="B12" s="42">
+        <v>0.05</v>
+      </c>
+      <c r="C12">
+        <v>3</v>
+      </c>
+      <c r="D12" s="40"/>
+      <c r="M12" s="20"/>
+      <c r="N12" s="42"/>
+    </row>
+    <row r="13" spans="1:14">
+      <c r="A13" t="s">
         <v>40</v>
       </c>
-      <c r="B12" s="20">
+      <c r="B13" s="42">
         <v>0.03</v>
       </c>
-      <c r="C12">
+      <c r="C13">
         <v>2</v>
       </c>
-    </row>
-    <row r="13" spans="1:12">
-      <c r="A13" t="s">
+      <c r="D13" s="40"/>
+      <c r="M13" s="20"/>
+      <c r="N13" s="42"/>
+    </row>
+    <row r="14" spans="1:14">
+      <c r="A14" t="s">
         <v>41</v>
       </c>
-      <c r="B13" s="20">
+      <c r="B14" s="42">
         <v>0.02</v>
       </c>
-      <c r="C13">
+      <c r="C14">
         <v>4</v>
       </c>
-    </row>
-    <row r="14" spans="1:12">
-      <c r="A14" t="s">
+      <c r="D14" s="40"/>
+      <c r="M14" s="20"/>
+      <c r="N14" s="42"/>
+    </row>
+    <row r="15" spans="1:14">
+      <c r="A15" t="s">
         <v>42</v>
       </c>
-      <c r="B14" s="20">
+      <c r="B15" s="42">
         <v>0.05</v>
       </c>
-      <c r="C14">
+      <c r="C15">
         <v>2</v>
       </c>
-    </row>
-    <row r="15" spans="1:12">
-      <c r="A15" t="s">
+      <c r="D15" s="40"/>
+      <c r="M15" s="20"/>
+      <c r="N15" s="42"/>
+    </row>
+    <row r="16" spans="1:14">
+      <c r="A16" t="s">
         <v>43</v>
       </c>
-      <c r="B15" s="20">
-        <v>0.05</v>
-      </c>
-      <c r="C15">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="16" spans="1:12">
-      <c r="A16" t="s">
-        <v>44</v>
-      </c>
-      <c r="B16" s="20">
+      <c r="B16" s="42">
         <v>0.05</v>
       </c>
       <c r="C16">
         <v>4</v>
       </c>
-    </row>
-    <row r="17" spans="1:3">
+      <c r="D16" s="40"/>
+      <c r="M16" s="20"/>
+      <c r="N16" s="42"/>
+    </row>
+    <row r="17" spans="1:14">
       <c r="A17" t="s">
+        <v>44</v>
+      </c>
+      <c r="B17" s="42">
+        <v>0.05</v>
+      </c>
+      <c r="C17">
+        <v>4</v>
+      </c>
+      <c r="D17" s="40"/>
+      <c r="M17" s="20"/>
+      <c r="N17" s="42"/>
+    </row>
+    <row r="18" spans="1:14">
+      <c r="A18" t="s">
         <v>45</v>
       </c>
-      <c r="B17" s="20">
-        <v>0.05</v>
-      </c>
-      <c r="C17">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3">
-      <c r="A18" t="s">
-        <v>46</v>
-      </c>
-      <c r="B18" s="20">
+      <c r="B18" s="42">
         <v>0.05</v>
       </c>
       <c r="C18">
         <v>2</v>
       </c>
-    </row>
-    <row r="19" spans="1:3">
+      <c r="D18" s="40"/>
+      <c r="M18" s="20"/>
+      <c r="N18" s="42"/>
+    </row>
+    <row r="19" spans="1:14">
       <c r="B19" s="22">
         <f>SUM(B2:B18)</f>
         <v>1.0000000000000002</v>
@@ -1426,4 +1637,301 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C3A3F4A-941E-4C2F-BC9A-D182D6DDCB37}">
+  <dimension ref="C2:N17"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.5"/>
+  <cols>
+    <col min="3" max="3" width="12" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.26953125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.54296875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="3:14">
+      <c r="C2" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="D2" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="E2" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="F2" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="G2" s="1"/>
+      <c r="I2" s="38" t="s">
+        <v>69</v>
+      </c>
+      <c r="J2" s="38"/>
+      <c r="K2" s="38"/>
+      <c r="L2" s="38"/>
+      <c r="M2" s="38"/>
+      <c r="N2" s="38"/>
+    </row>
+    <row r="3" spans="3:14">
+      <c r="C3" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="D3" s="10">
+        <v>3.9</v>
+      </c>
+      <c r="E3" s="35">
+        <v>3.6</v>
+      </c>
+      <c r="F3" s="9">
+        <v>3.84</v>
+      </c>
+      <c r="I3" s="38"/>
+      <c r="J3" s="38"/>
+      <c r="K3" s="38"/>
+      <c r="L3" s="38"/>
+      <c r="M3" s="38"/>
+      <c r="N3" s="38"/>
+    </row>
+    <row r="4" spans="3:14">
+      <c r="C4" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="D4" s="10">
+        <v>3.2</v>
+      </c>
+      <c r="E4" s="36">
+        <v>3.4</v>
+      </c>
+      <c r="F4" s="9">
+        <v>3.24</v>
+      </c>
+      <c r="I4" s="38"/>
+      <c r="J4" s="38"/>
+      <c r="K4" s="38"/>
+      <c r="L4" s="38"/>
+      <c r="M4" s="38"/>
+      <c r="N4" s="38"/>
+    </row>
+    <row r="5" spans="3:14">
+      <c r="C5" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="D5" s="34">
+        <v>2.4</v>
+      </c>
+      <c r="E5" s="10">
+        <v>4</v>
+      </c>
+      <c r="F5" s="9">
+        <v>2.72</v>
+      </c>
+      <c r="I5" s="38"/>
+      <c r="J5" s="38"/>
+      <c r="K5" s="38"/>
+      <c r="L5" s="38"/>
+      <c r="M5" s="38"/>
+      <c r="N5" s="38"/>
+    </row>
+    <row r="8" spans="3:14" ht="43.5">
+      <c r="C8" s="26" t="s">
+        <v>65</v>
+      </c>
+      <c r="D8" s="26" t="s">
+        <v>59</v>
+      </c>
+      <c r="E8" s="26" t="s">
+        <v>60</v>
+      </c>
+      <c r="F8" s="26" t="s">
+        <v>61</v>
+      </c>
+      <c r="G8" s="26" t="s">
+        <v>66</v>
+      </c>
+      <c r="I8" s="38" t="s">
+        <v>70</v>
+      </c>
+      <c r="J8" s="38"/>
+      <c r="K8" s="38"/>
+      <c r="L8" s="38"/>
+      <c r="M8" s="38"/>
+      <c r="N8" s="38"/>
+    </row>
+    <row r="9" spans="3:14">
+      <c r="C9" s="27" t="s">
+        <v>62</v>
+      </c>
+      <c r="D9" s="30">
+        <v>3.6</v>
+      </c>
+      <c r="E9" s="28">
+        <v>4</v>
+      </c>
+      <c r="F9" s="28">
+        <v>4</v>
+      </c>
+      <c r="G9" s="33">
+        <f>AVERAGE(D9:F9)</f>
+        <v>3.8666666666666667</v>
+      </c>
+      <c r="I9" s="38"/>
+      <c r="J9" s="38"/>
+      <c r="K9" s="38"/>
+      <c r="L9" s="38"/>
+      <c r="M9" s="38"/>
+      <c r="N9" s="38"/>
+    </row>
+    <row r="10" spans="3:14">
+      <c r="C10" s="27" t="s">
+        <v>63</v>
+      </c>
+      <c r="D10" s="28">
+        <v>4</v>
+      </c>
+      <c r="E10" s="31">
+        <v>3.4</v>
+      </c>
+      <c r="F10" s="28">
+        <v>3.9</v>
+      </c>
+      <c r="G10" s="33">
+        <f>AVERAGE(D10:F10)</f>
+        <v>3.7666666666666671</v>
+      </c>
+      <c r="I10" s="38"/>
+      <c r="J10" s="38"/>
+      <c r="K10" s="38"/>
+      <c r="L10" s="38"/>
+      <c r="M10" s="38"/>
+      <c r="N10" s="38"/>
+    </row>
+    <row r="11" spans="3:14">
+      <c r="C11" s="27" t="s">
+        <v>64</v>
+      </c>
+      <c r="D11" s="28">
+        <v>2.9</v>
+      </c>
+      <c r="E11" s="28">
+        <v>3</v>
+      </c>
+      <c r="F11" s="32">
+        <v>2.4</v>
+      </c>
+      <c r="G11" s="33">
+        <f>AVERAGE(D11:F11)</f>
+        <v>2.7666666666666671</v>
+      </c>
+    </row>
+    <row r="12" spans="3:14">
+      <c r="I12" s="21"/>
+    </row>
+    <row r="13" spans="3:14">
+      <c r="D13" s="22">
+        <v>0.8</v>
+      </c>
+      <c r="E13" s="22">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="14" spans="3:14">
+      <c r="C14" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="D14" s="29" t="s">
+        <v>55</v>
+      </c>
+      <c r="E14" s="19" t="s">
+        <v>67</v>
+      </c>
+      <c r="F14" s="19" t="s">
+        <v>68</v>
+      </c>
+      <c r="I14" s="39" t="s">
+        <v>71</v>
+      </c>
+      <c r="J14" s="39"/>
+      <c r="K14" s="39"/>
+      <c r="L14" s="39"/>
+      <c r="M14" s="39"/>
+      <c r="N14" s="39"/>
+    </row>
+    <row r="15" spans="3:14">
+      <c r="C15" s="27" t="s">
+        <v>49</v>
+      </c>
+      <c r="D15" s="29">
+        <f>D3</f>
+        <v>3.9</v>
+      </c>
+      <c r="E15" s="29">
+        <f>G9</f>
+        <v>3.8666666666666667</v>
+      </c>
+      <c r="F15" s="37">
+        <f>(D15*$D$13)+(E15*$E$13)</f>
+        <v>3.8933333333333335</v>
+      </c>
+      <c r="I15" s="39"/>
+      <c r="J15" s="39"/>
+      <c r="K15" s="39"/>
+      <c r="L15" s="39"/>
+      <c r="M15" s="39"/>
+      <c r="N15" s="39"/>
+    </row>
+    <row r="16" spans="3:14">
+      <c r="C16" s="27" t="s">
+        <v>50</v>
+      </c>
+      <c r="D16" s="29">
+        <f>D4</f>
+        <v>3.2</v>
+      </c>
+      <c r="E16" s="29">
+        <f>G10</f>
+        <v>3.7666666666666671</v>
+      </c>
+      <c r="F16" s="37">
+        <f>(D16*$D$13)+(E16*$E$13)</f>
+        <v>3.3133333333333339</v>
+      </c>
+      <c r="I16" s="39"/>
+      <c r="J16" s="39"/>
+      <c r="K16" s="39"/>
+      <c r="L16" s="39"/>
+      <c r="M16" s="39"/>
+      <c r="N16" s="39"/>
+    </row>
+    <row r="17" spans="3:14">
+      <c r="C17" s="27" t="s">
+        <v>51</v>
+      </c>
+      <c r="D17" s="29">
+        <f>D5</f>
+        <v>2.4</v>
+      </c>
+      <c r="E17" s="29">
+        <f>G11</f>
+        <v>2.7666666666666671</v>
+      </c>
+      <c r="F17" s="37">
+        <f>(D17*$D$13)+(E17*$E$13)</f>
+        <v>2.4733333333333336</v>
+      </c>
+      <c r="I17" s="39"/>
+      <c r="J17" s="39"/>
+      <c r="K17" s="39"/>
+      <c r="L17" s="39"/>
+      <c r="M17" s="39"/>
+      <c r="N17" s="39"/>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="I2:N5"/>
+    <mergeCell ref="I8:N10"/>
+    <mergeCell ref="I14:N17"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: Update HR analytics spreadsheet and remove temporary file
</commit_message>
<xml_diff>
--- a/Raquel_Pawnshop_HR_Workforce_Analytics_&_Evaluation _Platform-Computation.xlsx
+++ b/Raquel_Pawnshop_HR_Workforce_Analytics_&_Evaluation _Platform-Computation.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\Raquel_HRD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83062282-663D-4988-9AEF-66FA45862314}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC161CA8-8BB5-48E9-A46C-030F9067ACB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" activeTab="1" xr2:uid="{22A5745B-9E59-4E91-9FA4-3C7DB1ABBFEE}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" activeTab="2" xr2:uid="{22A5745B-9E59-4E91-9FA4-3C7DB1ABBFEE}"/>
   </bookViews>
   <sheets>
     <sheet name="auto" sheetId="1" r:id="rId1"/>
     <sheet name="manual" sheetId="2" r:id="rId2"/>
-    <sheet name="Sheet1" sheetId="4" r:id="rId3"/>
+    <sheet name="KRA" sheetId="6" r:id="rId3"/>
+    <sheet name="Behavior" sheetId="7" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -81,7 +82,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="79">
   <si>
     <t>Rating Scale</t>
   </si>
@@ -248,61 +249,85 @@
     <t>Miguel</t>
   </si>
   <si>
-    <t>kra score</t>
-  </si>
-  <si>
-    <t>self core behaviors</t>
-  </si>
-  <si>
-    <t>score</t>
-  </si>
-  <si>
-    <t>employee</t>
-  </si>
-  <si>
-    <t>HR Manager Rates</t>
-  </si>
-  <si>
-    <t>HR Supervisor Rates</t>
-  </si>
-  <si>
-    <t>HR Staff Rates</t>
-  </si>
-  <si>
-    <t>HR Manager</t>
-  </si>
-  <si>
-    <t>HR Supervisor</t>
-  </si>
-  <si>
-    <t>HR Staff</t>
-  </si>
-  <si>
-    <t>Employee Being Rated BAHAVIOR</t>
-  </si>
-  <si>
     <t>AVERAGE</t>
   </si>
   <si>
-    <t>peer 360 rating</t>
-  </si>
-  <si>
-    <t>final result/score</t>
-  </si>
-  <si>
-    <t xml:space="preserve">THIS IS THE INITIAL PROCESS FOR SELF RATING </t>
-  </si>
-  <si>
-    <t>THIS IS THE BEHAVIOR 360 RATING (PEERS)</t>
-  </si>
-  <si>
-    <t>THIS IS THE SYSTEM MUST ABSORBED</t>
+    <t>Criterion</t>
+  </si>
+  <si>
+    <t>Self-rating</t>
+  </si>
+  <si>
+    <t>Head-reviewed rating</t>
+  </si>
+  <si>
+    <t>Effective rating</t>
+  </si>
+  <si>
+    <t>Miguel Torres</t>
+  </si>
+  <si>
+    <t>Employee being rated</t>
+  </si>
+  <si>
+    <t>Rater</t>
+  </si>
+  <si>
+    <t>Type</t>
+  </si>
+  <si>
+    <t>Respect</t>
+  </si>
+  <si>
+    <t>Accountability</t>
+  </si>
+  <si>
+    <t>Commitment</t>
+  </si>
+  <si>
+    <t>Teamwork</t>
+  </si>
+  <si>
+    <t>Integrity</t>
+  </si>
+  <si>
+    <t>Self</t>
+  </si>
+  <si>
+    <t>Patricia Gomez</t>
+  </si>
+  <si>
+    <t>Department 360</t>
+  </si>
+  <si>
+    <t>Elena Delgado</t>
+  </si>
+  <si>
+    <t>Positive</t>
+  </si>
+  <si>
+    <t>Improvement</t>
+  </si>
+  <si>
+    <t>Client experience</t>
+  </si>
+  <si>
+    <t>KRA</t>
+  </si>
+  <si>
+    <t>Core Values &amp; Behaviors</t>
+  </si>
+  <si>
+    <t>TOTAL</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="165" formatCode="0.000"/>
+  </numFmts>
   <fonts count="9">
     <font>
       <sz val="11"/>
@@ -364,7 +389,7 @@
       <name val="Arial Unicode MS"/>
     </font>
   </fonts>
-  <fills count="12">
+  <fills count="13">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -406,25 +431,31 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.39997558519241921"/>
+        <fgColor theme="9"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="-0.249977111117893"/>
+        <fgColor theme="8" tint="0.39997558519241921"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.39997558519241921"/>
+        <fgColor theme="8"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.39997558519241921"/>
+        <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.39997558519241921"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -506,7 +537,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -578,47 +609,50 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="8" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="8" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="9" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="10" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="2" fontId="0" fillId="9" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="8" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="11" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1274,13 +1308,16 @@
   <dimension ref="A1:N19"/>
   <sheetFormatPr defaultColWidth="7" defaultRowHeight="14.5"/>
   <cols>
+    <col min="1" max="1" width="8.90625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="5.90625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="19.36328125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="5.90625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.08984375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.26953125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="17.54296875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="10" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="16.6328125" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="9.7265625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14">
@@ -1319,26 +1356,26 @@
       <c r="A2" t="s">
         <v>21</v>
       </c>
-      <c r="B2" s="42">
-        <v>0.05</v>
+      <c r="B2" s="28">
+        <v>0.3</v>
       </c>
       <c r="C2">
-        <v>2</v>
-      </c>
-      <c r="D2" s="40"/>
+        <v>4</v>
+      </c>
+      <c r="D2" s="27"/>
       <c r="E2" t="s">
         <v>22</v>
       </c>
       <c r="F2" s="24">
-        <v>4</v>
-      </c>
-      <c r="H2" s="41">
+        <v>1</v>
+      </c>
+      <c r="H2" s="29">
         <f>SUMPRODUCT(B2:B18,C2:C18)</f>
-        <v>3.3900000000000006</v>
-      </c>
-      <c r="I2" s="21">
+        <v>2.9000000000000004</v>
+      </c>
+      <c r="I2" s="31">
         <f>F10/8</f>
-        <v>3.125</v>
+        <v>3.375</v>
       </c>
       <c r="J2" s="22">
         <v>0.8</v>
@@ -1346,145 +1383,125 @@
       <c r="K2" s="22">
         <v>0.2</v>
       </c>
-      <c r="L2" s="21">
+      <c r="L2" s="30">
         <f>(H2*J2)+(I2*K2)</f>
-        <v>3.3370000000000006</v>
+        <v>2.9950000000000001</v>
       </c>
       <c r="M2" s="20"/>
-      <c r="N2" s="42"/>
+      <c r="N2" s="28"/>
     </row>
     <row r="3" spans="1:14">
       <c r="A3" t="s">
         <v>23</v>
       </c>
-      <c r="B3" s="42">
-        <v>0.1</v>
+      <c r="B3" s="28">
+        <v>0.3</v>
       </c>
       <c r="C3">
-        <v>3</v>
-      </c>
-      <c r="D3" s="40"/>
+        <v>1</v>
+      </c>
+      <c r="D3" s="27"/>
       <c r="E3" t="s">
         <v>24</v>
       </c>
       <c r="F3" s="24">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M3" s="20"/>
-      <c r="N3" s="42"/>
+      <c r="N3" s="28"/>
     </row>
     <row r="4" spans="1:14">
       <c r="A4" t="s">
         <v>25</v>
       </c>
-      <c r="B4" s="42">
-        <v>0.05</v>
+      <c r="B4" s="28">
+        <v>0.2</v>
       </c>
       <c r="C4">
-        <v>4</v>
-      </c>
-      <c r="D4" s="40"/>
+        <v>3</v>
+      </c>
+      <c r="D4" s="27"/>
       <c r="E4" t="s">
         <v>26</v>
       </c>
       <c r="F4" s="24">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I4" s="21"/>
       <c r="M4" s="20"/>
-      <c r="N4" s="42"/>
+      <c r="N4" s="28"/>
     </row>
     <row r="5" spans="1:14">
       <c r="A5" t="s">
         <v>27</v>
       </c>
-      <c r="B5" s="42">
-        <v>0.05</v>
+      <c r="B5" s="28">
+        <v>0.2</v>
       </c>
       <c r="C5">
-        <v>3</v>
-      </c>
-      <c r="D5" s="40"/>
+        <v>4</v>
+      </c>
+      <c r="D5" s="27"/>
       <c r="E5" t="s">
         <v>28</v>
       </c>
       <c r="F5" s="24">
-        <v>2</v>
-      </c>
-      <c r="M5" s="20"/>
-      <c r="N5" s="42"/>
+        <v>4</v>
+      </c>
+      <c r="I5" s="20"/>
+      <c r="J5" s="28"/>
     </row>
     <row r="6" spans="1:14">
       <c r="A6" t="s">
         <v>29</v>
       </c>
-      <c r="B6" s="42">
-        <v>0.05</v>
-      </c>
-      <c r="C6">
-        <v>4</v>
-      </c>
-      <c r="D6" s="40"/>
+      <c r="B6" s="28"/>
+      <c r="D6" s="27"/>
       <c r="E6" t="s">
         <v>30</v>
       </c>
       <c r="F6" s="24">
-        <v>2</v>
-      </c>
-      <c r="M6" s="20"/>
-      <c r="N6" s="42"/>
+        <v>4</v>
+      </c>
+      <c r="I6" s="20"/>
+      <c r="J6" s="28"/>
     </row>
     <row r="7" spans="1:14">
       <c r="A7" t="s">
         <v>31</v>
       </c>
-      <c r="B7" s="42">
-        <v>0.05</v>
-      </c>
-      <c r="C7">
-        <v>4</v>
-      </c>
-      <c r="D7" s="40"/>
+      <c r="B7" s="28"/>
+      <c r="D7" s="27"/>
       <c r="E7" t="s">
         <v>32</v>
       </c>
       <c r="F7" s="24">
-        <v>3</v>
-      </c>
-      <c r="M7" s="20"/>
-      <c r="N7" s="42"/>
+        <v>4</v>
+      </c>
+      <c r="I7" s="20"/>
+      <c r="J7" s="28"/>
     </row>
     <row r="8" spans="1:14">
       <c r="A8" t="s">
         <v>33</v>
       </c>
-      <c r="B8" s="42">
-        <v>0.2</v>
-      </c>
-      <c r="C8">
-        <v>4</v>
-      </c>
-      <c r="D8" s="40"/>
+      <c r="B8" s="28"/>
+      <c r="D8" s="27"/>
       <c r="E8" t="s">
         <v>34</v>
       </c>
       <c r="F8" s="24">
         <v>3</v>
       </c>
-      <c r="M8" s="20"/>
-      <c r="N8" s="42"/>
+      <c r="I8" s="20"/>
+      <c r="J8" s="28"/>
     </row>
     <row r="9" spans="1:14">
       <c r="A9" t="s">
         <v>35</v>
       </c>
-      <c r="B9" s="42">
-        <v>0.1</v>
-      </c>
-      <c r="C9">
-        <v>4</v>
-      </c>
-      <c r="D9" s="40"/>
+      <c r="B9" s="28"/>
+      <c r="D9" s="27"/>
       <c r="E9" t="s">
         <v>36</v>
       </c>
@@ -1492,146 +1509,102 @@
         <v>4</v>
       </c>
       <c r="M9" s="20"/>
-      <c r="N9" s="42"/>
+      <c r="N9" s="28"/>
     </row>
     <row r="10" spans="1:14">
       <c r="A10" t="s">
         <v>37</v>
       </c>
-      <c r="B10" s="42">
-        <v>0.02</v>
-      </c>
-      <c r="C10">
-        <v>3</v>
-      </c>
-      <c r="D10" s="40"/>
+      <c r="B10" s="28"/>
+      <c r="D10" s="27"/>
       <c r="F10" s="23">
         <f>SUM(F2:F9)</f>
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="M10" s="20"/>
-      <c r="N10" s="42"/>
+      <c r="N10" s="28"/>
     </row>
     <row r="11" spans="1:14">
       <c r="A11" t="s">
         <v>38</v>
       </c>
-      <c r="B11" s="42">
-        <v>0.03</v>
-      </c>
-      <c r="C11">
-        <v>3</v>
-      </c>
-      <c r="D11" s="40"/>
+      <c r="B11" s="28"/>
+      <c r="D11" s="27"/>
       <c r="M11" s="20"/>
-      <c r="N11" s="42"/>
+      <c r="N11" s="28"/>
     </row>
     <row r="12" spans="1:14">
       <c r="A12" t="s">
         <v>39</v>
       </c>
-      <c r="B12" s="42">
-        <v>0.05</v>
-      </c>
-      <c r="C12">
-        <v>3</v>
-      </c>
-      <c r="D12" s="40"/>
+      <c r="B12" s="28"/>
+      <c r="D12" s="27"/>
       <c r="M12" s="20"/>
-      <c r="N12" s="42"/>
+      <c r="N12" s="28"/>
     </row>
     <row r="13" spans="1:14">
       <c r="A13" t="s">
         <v>40</v>
       </c>
-      <c r="B13" s="42">
-        <v>0.03</v>
-      </c>
-      <c r="C13">
-        <v>2</v>
-      </c>
-      <c r="D13" s="40"/>
-      <c r="M13" s="20"/>
-      <c r="N13" s="42"/>
+      <c r="B13" s="28"/>
+      <c r="D13" s="27"/>
+      <c r="H13" s="20"/>
+      <c r="I13" s="28"/>
     </row>
     <row r="14" spans="1:14">
       <c r="A14" t="s">
         <v>41</v>
       </c>
-      <c r="B14" s="42">
-        <v>0.02</v>
-      </c>
-      <c r="C14">
-        <v>4</v>
-      </c>
-      <c r="D14" s="40"/>
-      <c r="M14" s="20"/>
-      <c r="N14" s="42"/>
+      <c r="B14" s="28"/>
+      <c r="D14" s="27"/>
+      <c r="H14" s="20"/>
+      <c r="I14" s="28"/>
+      <c r="K14" s="21"/>
     </row>
     <row r="15" spans="1:14">
       <c r="A15" t="s">
         <v>42</v>
       </c>
-      <c r="B15" s="42">
-        <v>0.05</v>
-      </c>
-      <c r="C15">
-        <v>2</v>
-      </c>
-      <c r="D15" s="40"/>
-      <c r="M15" s="20"/>
-      <c r="N15" s="42"/>
+      <c r="B15" s="28"/>
+      <c r="D15" s="27"/>
+      <c r="H15" s="20"/>
+      <c r="I15" s="28"/>
     </row>
     <row r="16" spans="1:14">
       <c r="A16" t="s">
         <v>43</v>
       </c>
-      <c r="B16" s="42">
-        <v>0.05</v>
-      </c>
-      <c r="C16">
-        <v>4</v>
-      </c>
-      <c r="D16" s="40"/>
-      <c r="M16" s="20"/>
-      <c r="N16" s="42"/>
-    </row>
-    <row r="17" spans="1:14">
+      <c r="B16" s="28"/>
+      <c r="D16" s="27"/>
+      <c r="H16" s="20"/>
+      <c r="I16" s="28"/>
+    </row>
+    <row r="17" spans="1:9">
       <c r="A17" t="s">
         <v>44</v>
       </c>
-      <c r="B17" s="42">
-        <v>0.05</v>
-      </c>
-      <c r="C17">
-        <v>4</v>
-      </c>
-      <c r="D17" s="40"/>
-      <c r="M17" s="20"/>
-      <c r="N17" s="42"/>
-    </row>
-    <row r="18" spans="1:14">
+      <c r="B17" s="28"/>
+      <c r="D17" s="27"/>
+      <c r="H17" s="20"/>
+      <c r="I17" s="28"/>
+    </row>
+    <row r="18" spans="1:9">
       <c r="A18" t="s">
         <v>45</v>
       </c>
-      <c r="B18" s="42">
-        <v>0.05</v>
-      </c>
-      <c r="C18">
-        <v>2</v>
-      </c>
-      <c r="D18" s="40"/>
-      <c r="M18" s="20"/>
-      <c r="N18" s="42"/>
-    </row>
-    <row r="19" spans="1:14">
+      <c r="B18" s="28"/>
+      <c r="D18" s="27"/>
+      <c r="H18" s="20"/>
+      <c r="I18" s="28"/>
+    </row>
+    <row r="19" spans="1:9">
       <c r="B19" s="22">
         <f>SUM(B2:B18)</f>
-        <v>1.0000000000000002</v>
+        <v>1</v>
       </c>
       <c r="C19" s="23">
         <f>SUM(C2:C18)</f>
-        <v>55</v>
+        <v>12</v>
       </c>
     </row>
   </sheetData>
@@ -1640,298 +1613,879 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C3A3F4A-941E-4C2F-BC9A-D182D6DDCB37}">
-  <dimension ref="C2:N17"/>
-  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.5"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{412713E5-6216-4E2A-886D-99615C42A4FD}">
+  <dimension ref="A1:N17"/>
+  <sheetFormatPr defaultColWidth="9.7265625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="3" max="3" width="12" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.26953125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.1796875" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.1796875" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="6.6328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.54296875" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.7265625" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.453125" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="7.54296875" style="1" customWidth="1"/>
+    <col min="8" max="8" width="13.1796875" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="6.08984375" style="1" customWidth="1"/>
+    <col min="10" max="10" width="21.08984375" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.453125" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.26953125" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="16384" width="9.7265625" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="3:14">
-      <c r="C2" s="9" t="s">
+    <row r="1" spans="1:14">
+      <c r="A1" s="26" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" s="26" t="s">
+        <v>56</v>
+      </c>
+      <c r="C1" s="26" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1" s="26" t="s">
+        <v>57</v>
+      </c>
+      <c r="E1" s="26" t="s">
         <v>58</v>
       </c>
-      <c r="D2" s="9" t="s">
+      <c r="F1" s="26" t="s">
+        <v>59</v>
+      </c>
+      <c r="H1" s="26" t="s">
+        <v>4</v>
+      </c>
+      <c r="I1" s="26" t="s">
+        <v>76</v>
+      </c>
+      <c r="J1" s="26" t="s">
+        <v>77</v>
+      </c>
+      <c r="K1" s="36" t="str">
+        <f>A7</f>
+        <v>Patricia Gomez</v>
+      </c>
+      <c r="L1" s="36" t="str">
+        <f>A12</f>
+        <v>Elena Delgado</v>
+      </c>
+      <c r="M1" s="36" t="s">
         <v>55</v>
       </c>
-      <c r="E2" s="9" t="s">
-        <v>56</v>
-      </c>
-      <c r="F2" s="9" t="s">
-        <v>57</v>
-      </c>
-      <c r="G2" s="1"/>
-      <c r="I2" s="38" t="s">
+      <c r="N1" s="36" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14">
+      <c r="A2" s="34" t="s">
+        <v>60</v>
+      </c>
+      <c r="B2" s="34" t="s">
+        <v>21</v>
+      </c>
+      <c r="C2" s="35">
+        <v>0.3</v>
+      </c>
+      <c r="D2" s="34">
+        <v>3</v>
+      </c>
+      <c r="E2" s="34">
+        <v>4</v>
+      </c>
+      <c r="F2" s="34">
+        <f>IF(D2="","",IF(E2="",D2,E2))</f>
+        <v>4</v>
+      </c>
+      <c r="H2" s="9" t="s">
+        <v>60</v>
+      </c>
+      <c r="I2" s="33">
+        <f>ROUND(SUMPRODUCT(C2:C5,F2:F5),3)</f>
+        <v>2.8</v>
+      </c>
+      <c r="J2" s="33">
+        <f>Behavior!M2</f>
+        <v>2.375</v>
+      </c>
+      <c r="K2" s="10">
+        <f>Behavior!M3</f>
+        <v>2.75</v>
+      </c>
+      <c r="L2" s="10">
+        <f>Behavior!M4</f>
+        <v>2</v>
+      </c>
+      <c r="M2" s="39">
+        <f>AVERAGE(J2:L2)</f>
+        <v>2.375</v>
+      </c>
+      <c r="N2" s="40">
+        <f>(I2*$G$17)+(M2*$H$17)</f>
+        <v>2.7149999999999999</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14">
+      <c r="A3" s="34" t="s">
+        <v>60</v>
+      </c>
+      <c r="B3" s="34" t="s">
+        <v>23</v>
+      </c>
+      <c r="C3" s="35">
+        <v>0.3</v>
+      </c>
+      <c r="D3" s="34">
+        <v>2</v>
+      </c>
+      <c r="E3" s="34">
+        <v>2</v>
+      </c>
+      <c r="F3" s="34">
+        <f t="shared" ref="F3:F5" si="0">IF(D3="","",IF(E3="",D3,E3))</f>
+        <v>2</v>
+      </c>
+      <c r="H3" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="I3" s="33">
+        <f>ROUND(SUMPRODUCT(C7:C10,F7:F10),3)</f>
+        <v>3.1</v>
+      </c>
+      <c r="K3" s="33">
+        <f>Behavior!M6</f>
+        <v>2.25</v>
+      </c>
+      <c r="L3" s="10">
+        <f>Behavior!M8</f>
+        <v>3</v>
+      </c>
+      <c r="M3" s="39">
+        <f t="shared" ref="M3:M4" si="1">AVERAGE(J3:L3)</f>
+        <v>2.625</v>
+      </c>
+      <c r="N3" s="40">
+        <f t="shared" ref="N3:N4" si="2">(I3*$G$17)+(M3*$H$17)</f>
+        <v>3.0050000000000003</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14">
+      <c r="A4" s="34" t="s">
+        <v>60</v>
+      </c>
+      <c r="B4" s="34" t="s">
+        <v>25</v>
+      </c>
+      <c r="C4" s="35">
+        <v>0.2</v>
+      </c>
+      <c r="D4" s="34">
+        <v>1</v>
+      </c>
+      <c r="E4" s="34">
+        <v>1</v>
+      </c>
+      <c r="F4" s="34">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="H4" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="I4" s="33">
+        <f>ROUND(SUMPRODUCT(C12:C15,F12:F15),3)</f>
+        <v>4</v>
+      </c>
+      <c r="K4" s="10">
+        <f>Behavior!M11</f>
+        <v>3.625</v>
+      </c>
+      <c r="L4" s="33">
+        <f>Behavior!M10</f>
+        <v>3.875</v>
+      </c>
+      <c r="M4" s="39">
+        <f t="shared" si="1"/>
+        <v>3.75</v>
+      </c>
+      <c r="N4" s="40">
+        <f t="shared" si="2"/>
+        <v>3.95</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14">
+      <c r="A5" s="34" t="s">
+        <v>60</v>
+      </c>
+      <c r="B5" s="34" t="s">
+        <v>27</v>
+      </c>
+      <c r="C5" s="35">
+        <v>0.2</v>
+      </c>
+      <c r="D5" s="34">
+        <v>2</v>
+      </c>
+      <c r="E5" s="34">
+        <v>4</v>
+      </c>
+      <c r="F5" s="34">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14">
+      <c r="A7" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="B7" s="34" t="s">
+        <v>21</v>
+      </c>
+      <c r="C7" s="35">
+        <v>0.3</v>
+      </c>
+      <c r="D7" s="9">
+        <v>3</v>
+      </c>
+      <c r="E7" s="9">
+        <v>4</v>
+      </c>
+      <c r="F7" s="34">
+        <f>IF(D7="","",IF(E7="",D7,E7))</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14">
+      <c r="A8" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="B8" s="34" t="s">
+        <v>23</v>
+      </c>
+      <c r="C8" s="35">
+        <v>0.3</v>
+      </c>
+      <c r="D8" s="9">
+        <v>3</v>
+      </c>
+      <c r="E8" s="9">
+        <v>3</v>
+      </c>
+      <c r="F8" s="34">
+        <f t="shared" ref="F8:F15" si="3">IF(D8="","",IF(E8="",D8,E8))</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14">
+      <c r="A9" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="B9" s="34" t="s">
+        <v>25</v>
+      </c>
+      <c r="C9" s="35">
+        <v>0.2</v>
+      </c>
+      <c r="D9" s="9">
+        <v>3</v>
+      </c>
+      <c r="E9" s="9">
+        <v>3</v>
+      </c>
+      <c r="F9" s="34">
+        <f t="shared" si="3"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14">
+      <c r="A10" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="B10" s="34" t="s">
+        <v>27</v>
+      </c>
+      <c r="C10" s="35">
+        <v>0.2</v>
+      </c>
+      <c r="D10" s="9">
+        <v>3</v>
+      </c>
+      <c r="E10" s="9">
+        <v>2</v>
+      </c>
+      <c r="F10" s="34">
+        <f t="shared" si="3"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14">
+      <c r="A12" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="B12" s="34" t="s">
+        <v>21</v>
+      </c>
+      <c r="C12" s="35">
+        <v>0.3</v>
+      </c>
+      <c r="D12" s="9">
+        <v>3</v>
+      </c>
+      <c r="E12" s="9">
+        <v>4</v>
+      </c>
+      <c r="F12" s="34">
+        <f t="shared" si="3"/>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14">
+      <c r="A13" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="B13" s="34" t="s">
+        <v>23</v>
+      </c>
+      <c r="C13" s="35">
+        <v>0.3</v>
+      </c>
+      <c r="D13" s="9">
+        <v>3</v>
+      </c>
+      <c r="E13" s="9">
+        <v>4</v>
+      </c>
+      <c r="F13" s="34">
+        <f t="shared" si="3"/>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14">
+      <c r="A14" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="B14" s="34" t="s">
+        <v>25</v>
+      </c>
+      <c r="C14" s="35">
+        <v>0.2</v>
+      </c>
+      <c r="D14" s="9">
+        <v>3</v>
+      </c>
+      <c r="E14" s="9">
+        <v>4</v>
+      </c>
+      <c r="F14" s="34">
+        <f t="shared" si="3"/>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14">
+      <c r="A15" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="B15" s="34" t="s">
+        <v>27</v>
+      </c>
+      <c r="C15" s="35">
+        <v>0.2</v>
+      </c>
+      <c r="D15" s="9">
+        <v>3</v>
+      </c>
+      <c r="E15" s="9">
+        <v>4</v>
+      </c>
+      <c r="F15" s="34">
+        <f t="shared" si="3"/>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="17" spans="7:8">
+      <c r="G17" s="37">
+        <v>0.8</v>
+      </c>
+      <c r="H17" s="37">
+        <v>0.2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E396ABDA-F64E-447D-9BAA-A4961C5442AD}">
+  <dimension ref="A1:N12"/>
+  <sheetFormatPr defaultColWidth="22" defaultRowHeight="14.5"/>
+  <cols>
+    <col min="1" max="1" width="18.90625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.1796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.08984375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="7.453125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="7.6328125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.08984375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.90625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.36328125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="7.7265625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="15.6328125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="6.54296875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14">
+      <c r="A1" s="26" t="s">
+        <v>61</v>
+      </c>
+      <c r="B1" s="26" t="s">
+        <v>62</v>
+      </c>
+      <c r="C1" s="26" t="s">
+        <v>63</v>
+      </c>
+      <c r="D1" s="26" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1" s="26" t="s">
+        <v>73</v>
+      </c>
+      <c r="F1" s="26" t="s">
+        <v>64</v>
+      </c>
+      <c r="G1" s="26" t="s">
+        <v>65</v>
+      </c>
+      <c r="H1" s="26" t="s">
+        <v>66</v>
+      </c>
+      <c r="I1" s="26" t="s">
+        <v>67</v>
+      </c>
+      <c r="J1" s="26" t="s">
+        <v>68</v>
+      </c>
+      <c r="K1" s="26" t="s">
+        <v>74</v>
+      </c>
+      <c r="L1" s="26" t="s">
+        <v>75</v>
+      </c>
+      <c r="M1" s="1"/>
+      <c r="N1" s="32" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14">
+      <c r="A2" s="34" t="s">
+        <v>60</v>
+      </c>
+      <c r="B2" s="34" t="s">
+        <v>60</v>
+      </c>
+      <c r="C2" s="34" t="s">
         <v>69</v>
       </c>
-      <c r="J2" s="38"/>
-      <c r="K2" s="38"/>
-      <c r="L2" s="38"/>
-      <c r="M2" s="38"/>
-      <c r="N2" s="38"/>
-    </row>
-    <row r="3" spans="3:14">
-      <c r="C3" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="D3" s="10">
-        <v>3.9</v>
-      </c>
-      <c r="E3" s="35">
-        <v>3.6</v>
-      </c>
-      <c r="F3" s="9">
-        <v>3.84</v>
-      </c>
-      <c r="I3" s="38"/>
-      <c r="J3" s="38"/>
-      <c r="K3" s="38"/>
-      <c r="L3" s="38"/>
-      <c r="M3" s="38"/>
-      <c r="N3" s="38"/>
-    </row>
-    <row r="4" spans="3:14">
-      <c r="C4" s="9" t="s">
-        <v>50</v>
-      </c>
-      <c r="D4" s="10">
-        <v>3.2</v>
-      </c>
-      <c r="E4" s="36">
-        <v>3.4</v>
-      </c>
-      <c r="F4" s="9">
-        <v>3.24</v>
-      </c>
-      <c r="I4" s="38"/>
-      <c r="J4" s="38"/>
-      <c r="K4" s="38"/>
-      <c r="L4" s="38"/>
-      <c r="M4" s="38"/>
-      <c r="N4" s="38"/>
-    </row>
-    <row r="5" spans="3:14">
-      <c r="C5" s="9" t="s">
-        <v>51</v>
-      </c>
-      <c r="D5" s="34">
-        <v>2.4</v>
-      </c>
-      <c r="E5" s="10">
-        <v>4</v>
-      </c>
-      <c r="F5" s="9">
-        <v>2.72</v>
-      </c>
-      <c r="I5" s="38"/>
-      <c r="J5" s="38"/>
-      <c r="K5" s="38"/>
-      <c r="L5" s="38"/>
-      <c r="M5" s="38"/>
-      <c r="N5" s="38"/>
-    </row>
-    <row r="8" spans="3:14" ht="43.5">
-      <c r="C8" s="26" t="s">
-        <v>65</v>
-      </c>
-      <c r="D8" s="26" t="s">
-        <v>59</v>
-      </c>
-      <c r="E8" s="26" t="s">
+      <c r="D2" s="42" t="s">
+        <v>54</v>
+      </c>
+      <c r="E2" s="34">
+        <v>4</v>
+      </c>
+      <c r="F2" s="34">
+        <v>2</v>
+      </c>
+      <c r="G2" s="34">
+        <v>1</v>
+      </c>
+      <c r="H2" s="34">
+        <v>2</v>
+      </c>
+      <c r="I2" s="34">
+        <v>3</v>
+      </c>
+      <c r="J2" s="34">
+        <v>2</v>
+      </c>
+      <c r="K2" s="34">
+        <v>1</v>
+      </c>
+      <c r="L2" s="34">
+        <v>4</v>
+      </c>
+      <c r="M2" s="25">
+        <f>IF(COUNT(E2:L2)=8,AVERAGE(E2:L2),"")</f>
+        <v>2.375</v>
+      </c>
+      <c r="N2" s="38">
+        <f>AVERAGE(M2:M4)</f>
+        <v>2.375</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14">
+      <c r="A3" s="34" t="s">
         <v>60</v>
       </c>
-      <c r="F8" s="26" t="s">
-        <v>61</v>
-      </c>
-      <c r="G8" s="26" t="s">
-        <v>66</v>
-      </c>
-      <c r="I8" s="38" t="s">
+      <c r="B3" s="34" t="s">
         <v>70</v>
       </c>
-      <c r="J8" s="38"/>
-      <c r="K8" s="38"/>
-      <c r="L8" s="38"/>
-      <c r="M8" s="38"/>
-      <c r="N8" s="38"/>
-    </row>
-    <row r="9" spans="3:14">
-      <c r="C9" s="27" t="s">
-        <v>62</v>
-      </c>
-      <c r="D9" s="30">
-        <v>3.6</v>
-      </c>
-      <c r="E9" s="28">
-        <v>4</v>
-      </c>
-      <c r="F9" s="28">
-        <v>4</v>
-      </c>
-      <c r="G9" s="33">
-        <f>AVERAGE(D9:F9)</f>
-        <v>3.8666666666666667</v>
-      </c>
-      <c r="I9" s="38"/>
-      <c r="J9" s="38"/>
-      <c r="K9" s="38"/>
-      <c r="L9" s="38"/>
-      <c r="M9" s="38"/>
-      <c r="N9" s="38"/>
-    </row>
-    <row r="10" spans="3:14">
-      <c r="C10" s="27" t="s">
-        <v>63</v>
-      </c>
-      <c r="D10" s="28">
-        <v>4</v>
-      </c>
-      <c r="E10" s="31">
-        <v>3.4</v>
-      </c>
-      <c r="F10" s="28">
-        <v>3.9</v>
-      </c>
-      <c r="G10" s="33">
-        <f>AVERAGE(D10:F10)</f>
-        <v>3.7666666666666671</v>
-      </c>
-      <c r="I10" s="38"/>
-      <c r="J10" s="38"/>
-      <c r="K10" s="38"/>
-      <c r="L10" s="38"/>
-      <c r="M10" s="38"/>
-      <c r="N10" s="38"/>
-    </row>
-    <row r="11" spans="3:14">
-      <c r="C11" s="27" t="s">
-        <v>64</v>
-      </c>
-      <c r="D11" s="28">
-        <v>2.9</v>
-      </c>
-      <c r="E11" s="28">
-        <v>3</v>
-      </c>
-      <c r="F11" s="32">
-        <v>2.4</v>
-      </c>
-      <c r="G11" s="33">
-        <f>AVERAGE(D11:F11)</f>
-        <v>2.7666666666666671</v>
-      </c>
-    </row>
-    <row r="12" spans="3:14">
-      <c r="I12" s="21"/>
-    </row>
-    <row r="13" spans="3:14">
-      <c r="D13" s="22">
-        <v>0.8</v>
-      </c>
-      <c r="E13" s="22">
-        <v>0.2</v>
-      </c>
-    </row>
-    <row r="14" spans="3:14">
-      <c r="C14" s="9" t="s">
-        <v>58</v>
-      </c>
-      <c r="D14" s="29" t="s">
-        <v>55</v>
-      </c>
-      <c r="E14" s="19" t="s">
-        <v>67</v>
-      </c>
-      <c r="F14" s="19" t="s">
-        <v>68</v>
-      </c>
-      <c r="I14" s="39" t="s">
+      <c r="C3" s="34" t="s">
         <v>71</v>
       </c>
-      <c r="J14" s="39"/>
-      <c r="K14" s="39"/>
-      <c r="L14" s="39"/>
-      <c r="M14" s="39"/>
-      <c r="N14" s="39"/>
-    </row>
-    <row r="15" spans="3:14">
-      <c r="C15" s="27" t="s">
-        <v>49</v>
-      </c>
-      <c r="D15" s="29">
-        <f>D3</f>
-        <v>3.9</v>
-      </c>
-      <c r="E15" s="29">
-        <f>G9</f>
-        <v>3.8666666666666667</v>
-      </c>
-      <c r="F15" s="37">
-        <f>(D15*$D$13)+(E15*$E$13)</f>
-        <v>3.8933333333333335</v>
-      </c>
-      <c r="I15" s="39"/>
-      <c r="J15" s="39"/>
-      <c r="K15" s="39"/>
-      <c r="L15" s="39"/>
-      <c r="M15" s="39"/>
-      <c r="N15" s="39"/>
-    </row>
-    <row r="16" spans="3:14">
-      <c r="C16" s="27" t="s">
-        <v>50</v>
-      </c>
-      <c r="D16" s="29">
-        <f>D4</f>
-        <v>3.2</v>
-      </c>
-      <c r="E16" s="29">
-        <f>G10</f>
-        <v>3.7666666666666671</v>
-      </c>
-      <c r="F16" s="37">
-        <f>(D16*$D$13)+(E16*$E$13)</f>
-        <v>3.3133333333333339</v>
-      </c>
-      <c r="I16" s="39"/>
-      <c r="J16" s="39"/>
-      <c r="K16" s="39"/>
-      <c r="L16" s="39"/>
-      <c r="M16" s="39"/>
-      <c r="N16" s="39"/>
-    </row>
-    <row r="17" spans="3:14">
-      <c r="C17" s="27" t="s">
-        <v>51</v>
-      </c>
-      <c r="D17" s="29">
-        <f>D5</f>
-        <v>2.4</v>
-      </c>
-      <c r="E17" s="29">
-        <f>G11</f>
-        <v>2.7666666666666671</v>
-      </c>
-      <c r="F17" s="37">
-        <f>(D17*$D$13)+(E17*$E$13)</f>
-        <v>2.4733333333333336</v>
-      </c>
-      <c r="I17" s="39"/>
-      <c r="J17" s="39"/>
-      <c r="K17" s="39"/>
-      <c r="L17" s="39"/>
-      <c r="M17" s="39"/>
-      <c r="N17" s="39"/>
+      <c r="D3" s="43" t="s">
+        <v>53</v>
+      </c>
+      <c r="E3" s="34">
+        <v>4</v>
+      </c>
+      <c r="F3" s="34">
+        <v>2</v>
+      </c>
+      <c r="G3" s="34">
+        <v>4</v>
+      </c>
+      <c r="H3" s="34">
+        <v>2</v>
+      </c>
+      <c r="I3" s="34">
+        <v>3</v>
+      </c>
+      <c r="J3" s="34">
+        <v>2</v>
+      </c>
+      <c r="K3" s="34">
+        <v>1</v>
+      </c>
+      <c r="L3" s="34">
+        <v>4</v>
+      </c>
+      <c r="M3" s="25">
+        <f t="shared" ref="I3:M12" si="0">IF(COUNT(E3:L3)=8,AVERAGE(E3:L3),"")</f>
+        <v>2.75</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14">
+      <c r="A4" s="34" t="s">
+        <v>60</v>
+      </c>
+      <c r="B4" s="34" t="s">
+        <v>72</v>
+      </c>
+      <c r="C4" s="34" t="s">
+        <v>71</v>
+      </c>
+      <c r="D4" s="41" t="s">
+        <v>52</v>
+      </c>
+      <c r="E4" s="34">
+        <v>1</v>
+      </c>
+      <c r="F4" s="34">
+        <v>2</v>
+      </c>
+      <c r="G4" s="34">
+        <v>1</v>
+      </c>
+      <c r="H4" s="34">
+        <v>2</v>
+      </c>
+      <c r="I4" s="34">
+        <v>3</v>
+      </c>
+      <c r="J4" s="34">
+        <v>2</v>
+      </c>
+      <c r="K4" s="34">
+        <v>1</v>
+      </c>
+      <c r="L4" s="34">
+        <v>4</v>
+      </c>
+      <c r="M4" s="25">
+        <f>IF(COUNT(E4:L4)=8,AVERAGE(E4:L4),"")</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14">
+      <c r="A5" s="1"/>
+      <c r="B5" s="1"/>
+      <c r="C5" s="1"/>
+      <c r="D5" s="1"/>
+    </row>
+    <row r="6" spans="1:14">
+      <c r="A6" s="34" t="s">
+        <v>70</v>
+      </c>
+      <c r="B6" s="34" t="s">
+        <v>70</v>
+      </c>
+      <c r="C6" s="34" t="s">
+        <v>69</v>
+      </c>
+      <c r="D6" s="43" t="s">
+        <v>53</v>
+      </c>
+      <c r="E6" s="9">
+        <v>1</v>
+      </c>
+      <c r="F6" s="9">
+        <v>3</v>
+      </c>
+      <c r="G6" s="9">
+        <v>2</v>
+      </c>
+      <c r="H6" s="9">
+        <v>1</v>
+      </c>
+      <c r="I6" s="9">
+        <v>3</v>
+      </c>
+      <c r="J6" s="9">
+        <v>3</v>
+      </c>
+      <c r="K6" s="9">
+        <v>2</v>
+      </c>
+      <c r="L6" s="9">
+        <v>3</v>
+      </c>
+      <c r="M6" s="1">
+        <f t="shared" si="0"/>
+        <v>2.25</v>
+      </c>
+      <c r="N6" s="38">
+        <f>AVERAGE(M6:M8)</f>
+        <v>2.625</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14">
+      <c r="A7" s="34" t="s">
+        <v>70</v>
+      </c>
+      <c r="B7" s="34" t="s">
+        <v>60</v>
+      </c>
+      <c r="C7" s="34" t="s">
+        <v>71</v>
+      </c>
+      <c r="D7" s="42" t="s">
+        <v>54</v>
+      </c>
+      <c r="E7" s="9">
+        <v>1</v>
+      </c>
+      <c r="F7" s="9">
+        <v>3</v>
+      </c>
+      <c r="G7" s="9">
+        <v>2</v>
+      </c>
+      <c r="H7" s="9">
+        <v>4</v>
+      </c>
+      <c r="I7" s="9">
+        <v>3</v>
+      </c>
+      <c r="J7" s="9">
+        <v>3</v>
+      </c>
+      <c r="K7" s="9">
+        <v>2</v>
+      </c>
+      <c r="L7" s="9">
+        <v>3</v>
+      </c>
+      <c r="M7" s="25">
+        <f t="shared" si="0"/>
+        <v>2.625</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14">
+      <c r="A8" s="34" t="s">
+        <v>70</v>
+      </c>
+      <c r="B8" s="34" t="s">
+        <v>72</v>
+      </c>
+      <c r="C8" s="34" t="s">
+        <v>71</v>
+      </c>
+      <c r="D8" s="41" t="s">
+        <v>52</v>
+      </c>
+      <c r="E8" s="9">
+        <v>4</v>
+      </c>
+      <c r="F8" s="9">
+        <v>3</v>
+      </c>
+      <c r="G8" s="9">
+        <v>2</v>
+      </c>
+      <c r="H8" s="9">
+        <v>4</v>
+      </c>
+      <c r="I8" s="9">
+        <v>3</v>
+      </c>
+      <c r="J8" s="9">
+        <v>3</v>
+      </c>
+      <c r="K8" s="9">
+        <v>2</v>
+      </c>
+      <c r="L8" s="9">
+        <v>3</v>
+      </c>
+      <c r="M8" s="25">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14">
+      <c r="A9" s="1"/>
+      <c r="B9" s="1"/>
+      <c r="C9" s="1"/>
+      <c r="D9" s="1"/>
+      <c r="E9" s="1"/>
+      <c r="F9" s="1"/>
+      <c r="G9" s="1"/>
+      <c r="H9" s="1"/>
+      <c r="I9" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+    </row>
+    <row r="10" spans="1:14">
+      <c r="A10" s="34" t="s">
+        <v>72</v>
+      </c>
+      <c r="B10" s="34" t="s">
+        <v>72</v>
+      </c>
+      <c r="C10" s="34" t="s">
+        <v>69</v>
+      </c>
+      <c r="D10" s="41" t="s">
+        <v>52</v>
+      </c>
+      <c r="E10" s="9">
+        <v>4</v>
+      </c>
+      <c r="F10" s="9">
+        <v>4</v>
+      </c>
+      <c r="G10" s="9">
+        <v>3</v>
+      </c>
+      <c r="H10" s="9">
+        <v>4</v>
+      </c>
+      <c r="I10" s="9">
+        <v>4</v>
+      </c>
+      <c r="J10" s="9">
+        <v>4</v>
+      </c>
+      <c r="K10" s="9">
+        <v>4</v>
+      </c>
+      <c r="L10" s="9">
+        <v>4</v>
+      </c>
+      <c r="M10" s="25">
+        <f t="shared" si="0"/>
+        <v>3.875</v>
+      </c>
+      <c r="N10" s="38">
+        <f>AVERAGE(M10:M12)</f>
+        <v>3.6666666666666665</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14">
+      <c r="A11" s="34" t="s">
+        <v>72</v>
+      </c>
+      <c r="B11" s="34" t="s">
+        <v>70</v>
+      </c>
+      <c r="C11" s="34" t="s">
+        <v>71</v>
+      </c>
+      <c r="D11" s="43" t="s">
+        <v>53</v>
+      </c>
+      <c r="E11" s="9">
+        <v>4</v>
+      </c>
+      <c r="F11" s="9">
+        <v>4</v>
+      </c>
+      <c r="G11" s="9">
+        <v>3</v>
+      </c>
+      <c r="H11" s="9">
+        <v>2</v>
+      </c>
+      <c r="I11" s="9">
+        <v>4</v>
+      </c>
+      <c r="J11" s="9">
+        <v>4</v>
+      </c>
+      <c r="K11" s="9">
+        <v>4</v>
+      </c>
+      <c r="L11" s="9">
+        <v>4</v>
+      </c>
+      <c r="M11" s="25">
+        <f t="shared" si="0"/>
+        <v>3.625</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14">
+      <c r="A12" s="34" t="s">
+        <v>72</v>
+      </c>
+      <c r="B12" s="34" t="s">
+        <v>60</v>
+      </c>
+      <c r="C12" s="34" t="s">
+        <v>71</v>
+      </c>
+      <c r="D12" s="42" t="s">
+        <v>54</v>
+      </c>
+      <c r="E12" s="9">
+        <v>4</v>
+      </c>
+      <c r="F12" s="9">
+        <v>4</v>
+      </c>
+      <c r="G12" s="9">
+        <v>3</v>
+      </c>
+      <c r="H12" s="9">
+        <v>1</v>
+      </c>
+      <c r="I12" s="9">
+        <v>4</v>
+      </c>
+      <c r="J12" s="9">
+        <v>4</v>
+      </c>
+      <c r="K12" s="9">
+        <v>4</v>
+      </c>
+      <c r="L12" s="9">
+        <v>4</v>
+      </c>
+      <c r="M12" s="25">
+        <f t="shared" si="0"/>
+        <v>3.5</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="I2:N5"/>
-    <mergeCell ref="I8:N10"/>
-    <mergeCell ref="I14:N17"/>
-  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>